<commit_message>
Publish restored P&L footer and frozen column headers
</commit_message>
<xml_diff>
--- a/public/checkmi/templates/车型损益表_空白公式模板.xlsx
+++ b/public/checkmi/templates/车型损益表_空白公式模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="车型损益表" sheetId="1" r:id="R1e537fb93b9b47f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="车型损益表" sheetId="1" r:id="R975330b25d194103"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,11 +13,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="0.0%"/>
     <numFmt numFmtId="177" formatCode="#,##0.0"/>
+    <numFmt numFmtId="178" formatCode="General"/>
+    <numFmt numFmtId="179" formatCode="#,##0;[Red](#,##0);–"/>
+    <numFmt numFmtId="180" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="49">
+  <fonts count="57">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -385,8 +388,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF31382E"/>
+      <name val="等线"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF31382E"/>
+      <name val="宋体"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF8C9188"/>
+      <name val="等线"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF383931"/>
+      <name val="微软雅黑"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF666B62"/>
+      <name val="等线"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF383931"/>
+      <name val="微软雅黑"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF215EA8"/>
+      <name val="微软雅黑"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF74766B"/>
+      <name val="微软雅黑"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -459,8 +504,21 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1EFE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF9E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="141">
+  <borders count="142">
     <border>
       <left/>
       <right/>
@@ -2202,11 +2260,13 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="141"/>
   </cellStyleXfs>
-  <cellXfs count="995">
+  <cellXfs count="1007">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -5165,6 +5225,42 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="50" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="50" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="176" fontId="51" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="49" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="52" fillId="16" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="54" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="55" fillId="17" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="180" fontId="49" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="17" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="178" fontId="56" fillId="15" borderId="141" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -23329,2317 +23425,2317 @@
       </c>
       <c s="335" r="DG69"/>
     </row>
-    <row r="70" spans="1:111" ht="22" customHeight="1">
-      <c s="321" r="A70"/>
-      <c s="322" r="B70"/>
-      <c s="331" r="C70"/>
-      <c s="332" r="D70"/>
-      <c s="332" r="E70"/>
-      <c s="333" r="F70"/>
-      <c s="332" r="G70"/>
-      <c s="332" r="H70"/>
-      <c s="333" r="I70"/>
-      <c s="332" r="J70"/>
-      <c s="332" r="K70"/>
-      <c s="333" r="L70"/>
-      <c s="332" r="M70"/>
-      <c s="332" r="N70"/>
-      <c s="333" r="O70"/>
-      <c s="332" r="P70"/>
-      <c s="332" r="Q70"/>
-      <c s="334" r="R70"/>
-      <c s="332" r="S70"/>
-      <c s="332" r="T70"/>
-      <c s="324" r="U70"/>
-      <c s="332" r="V70"/>
-      <c s="332" r="W70"/>
-      <c s="333" r="X70"/>
-      <c s="332" r="Y70"/>
-      <c s="332" r="Z70"/>
-      <c s="333" r="AA70"/>
-      <c s="332" r="AB70"/>
-      <c s="332" r="AC70"/>
-      <c s="333" r="AD70"/>
-      <c s="332" r="AE70"/>
-      <c s="332" r="AF70"/>
-      <c s="333" r="AG70"/>
-      <c s="332" r="AH70"/>
-      <c s="332" r="AI70"/>
-      <c s="334" r="AJ70"/>
-      <c s="332" r="AK70"/>
-      <c s="332" r="AL70"/>
-      <c s="324" r="AM70"/>
-      <c s="332" r="AN70"/>
-      <c s="332" r="AO70"/>
-      <c s="333" r="AP70"/>
-      <c s="332" r="AQ70"/>
-      <c s="332" r="AR70"/>
-      <c s="333" r="AS70"/>
-      <c s="332" r="AT70"/>
-      <c s="332" r="AU70"/>
-      <c s="333" r="AV70"/>
-      <c s="332" r="AW70"/>
-      <c s="332" r="AX70"/>
-      <c s="333" r="AY70"/>
-      <c s="332" r="AZ70"/>
-      <c s="332" r="BA70"/>
-      <c s="334" r="BB70"/>
-      <c s="332" r="BC70"/>
-      <c s="332" r="BD70"/>
-      <c s="324" r="BE70"/>
-      <c s="332" r="BF70"/>
-      <c s="332" r="BG70"/>
-      <c s="333" r="BH70"/>
-      <c s="332" r="BI70"/>
-      <c s="332" r="BJ70"/>
-      <c s="333" r="BK70"/>
-      <c s="332" r="BL70"/>
-      <c s="332" r="BM70"/>
-      <c s="333" r="BN70"/>
-      <c s="332" r="BO70"/>
-      <c s="332" r="BP70"/>
-      <c s="333" r="BQ70"/>
-      <c s="332" r="BR70"/>
-      <c s="332" r="BS70"/>
-      <c s="334" r="BT70"/>
-      <c s="332" r="BU70"/>
-      <c s="332" r="BV70"/>
-      <c s="324" r="BW70"/>
-      <c s="332" r="BX70"/>
-      <c s="332" r="BY70"/>
-      <c s="333" r="BZ70"/>
-      <c s="332" r="CA70"/>
-      <c s="332" r="CB70"/>
-      <c s="333" r="CC70"/>
-      <c s="332" r="CD70"/>
-      <c s="332" r="CE70"/>
-      <c s="333" r="CF70"/>
-      <c s="332" r="CG70"/>
-      <c s="332" r="CH70"/>
-      <c s="333" r="CI70"/>
-      <c s="332" r="CJ70"/>
-      <c s="332" r="CK70"/>
-      <c s="334" r="CL70"/>
-      <c s="332" r="CM70"/>
-      <c s="332" r="CN70"/>
-      <c s="325" r="CO70"/>
-      <c s="332" r="CP70"/>
-      <c s="332" r="CQ70"/>
-      <c s="326" r="CR70"/>
-      <c s="332" r="CS70"/>
-      <c s="332" r="CT70"/>
-      <c s="326" r="CU70"/>
-      <c s="332" r="CV70"/>
-      <c s="332" r="CW70"/>
-      <c s="326" r="CX70"/>
-      <c s="332" r="CY70"/>
-      <c s="332" r="CZ70"/>
-      <c s="326" r="DA70"/>
-      <c s="332" r="DB70"/>
-      <c s="332" r="DC70"/>
-      <c s="326" r="DD70"/>
-      <c s="332" r="DE70"/>
-      <c s="332" r="DF70"/>
-      <c s="335" r="DG70"/>
+    <row r="70" ht="22" customHeight="1">
+      <c s="995" r="A70"/>
+      <c s="996" r="B70"/>
+      <c s="995" r="C70"/>
+      <c s="997" r="D70"/>
+      <c s="998" r="E70"/>
+      <c s="995" r="F70"/>
+      <c s="997" r="G70"/>
+      <c s="998" r="H70"/>
+      <c s="995" r="I70"/>
+      <c s="997" r="J70"/>
+      <c s="998" r="K70"/>
+      <c s="995" r="L70"/>
+      <c s="997" r="M70"/>
+      <c s="998" r="N70"/>
+      <c s="995" r="O70"/>
+      <c s="997" r="P70"/>
+      <c s="998" r="Q70"/>
+      <c s="995" r="R70"/>
+      <c s="999" r="S70"/>
+      <c s="998" r="T70"/>
+      <c s="995" r="U70"/>
+      <c s="997" r="V70"/>
+      <c s="998" r="W70"/>
+      <c s="995" r="X70"/>
+      <c s="997" r="Y70"/>
+      <c s="998" r="Z70"/>
+      <c s="995" r="AA70"/>
+      <c s="997" r="AB70"/>
+      <c s="998" r="AC70"/>
+      <c s="995" r="AD70"/>
+      <c s="997" r="AE70"/>
+      <c s="998" r="AF70"/>
+      <c s="995" r="AG70"/>
+      <c s="997" r="AH70"/>
+      <c s="998" r="AI70"/>
+      <c s="995" r="AJ70"/>
+      <c s="999" r="AK70"/>
+      <c s="998" r="AL70"/>
+      <c s="995" r="AM70"/>
+      <c s="997" r="AN70"/>
+      <c s="998" r="AO70"/>
+      <c s="995" r="AP70"/>
+      <c s="997" r="AQ70"/>
+      <c s="998" r="AR70"/>
+      <c s="995" r="AS70"/>
+      <c s="997" r="AT70"/>
+      <c s="998" r="AU70"/>
+      <c s="995" r="AV70"/>
+      <c s="997" r="AW70"/>
+      <c s="998" r="AX70"/>
+      <c s="995" r="AY70"/>
+      <c s="997" r="AZ70"/>
+      <c s="998" r="BA70"/>
+      <c s="995" r="BB70"/>
+      <c s="999" r="BC70"/>
+      <c s="998" r="BD70"/>
+      <c s="995" r="BE70"/>
+      <c s="997" r="BF70"/>
+      <c s="998" r="BG70"/>
+      <c s="995" r="BH70"/>
+      <c s="997" r="BI70"/>
+      <c s="998" r="BJ70"/>
+      <c s="995" r="BK70"/>
+      <c s="997" r="BL70"/>
+      <c s="998" r="BM70"/>
+      <c s="995" r="BN70"/>
+      <c s="997" r="BO70"/>
+      <c s="998" r="BP70"/>
+      <c s="995" r="BQ70"/>
+      <c s="997" r="BR70"/>
+      <c s="998" r="BS70"/>
+      <c s="995" r="BT70"/>
+      <c s="999" r="BU70"/>
+      <c s="998" r="BV70"/>
+      <c s="995" r="BW70"/>
+      <c s="997" r="BX70"/>
+      <c s="998" r="BY70"/>
+      <c s="995" r="BZ70"/>
+      <c s="997" r="CA70"/>
+      <c s="998" r="CB70"/>
+      <c s="995" r="CC70"/>
+      <c s="997" r="CD70"/>
+      <c s="998" r="CE70"/>
+      <c s="995" r="CF70"/>
+      <c s="997" r="CG70"/>
+      <c s="998" r="CH70"/>
+      <c s="995" r="CI70"/>
+      <c s="997" r="CJ70"/>
+      <c s="998" r="CK70"/>
+      <c s="995" r="CL70"/>
+      <c s="999" r="CM70"/>
+      <c s="998" r="CN70"/>
+      <c s="995" r="CO70"/>
+      <c s="999" r="CP70"/>
+      <c s="998" r="CQ70"/>
+      <c s="995" r="CR70"/>
+      <c s="999" r="CS70"/>
+      <c s="998" r="CT70"/>
+      <c s="995" r="CU70"/>
+      <c s="999" r="CV70"/>
+      <c s="998" r="CW70"/>
+      <c s="995" r="CX70"/>
+      <c s="999" r="CY70"/>
+      <c s="998" r="CZ70"/>
+      <c s="995" r="DA70"/>
+      <c s="999" r="DB70"/>
+      <c s="998" r="DC70"/>
+      <c s="995" r="DD70"/>
+      <c s="999" r="DE70"/>
+      <c s="998" r="DF70"/>
+      <c s="995" r="DG70"/>
     </row>
-    <row r="71" spans="1:111" ht="22" customHeight="1">
-      <c s="321" r="A71"/>
-      <c s="322" r="B71"/>
-      <c s="331" r="C71"/>
-      <c s="332" r="D71"/>
-      <c s="332" r="E71"/>
-      <c s="333" r="F71"/>
-      <c s="332" r="G71"/>
-      <c s="332" r="H71"/>
-      <c s="333" r="I71"/>
-      <c s="332" r="J71"/>
-      <c s="332" r="K71"/>
-      <c s="333" r="L71"/>
-      <c s="332" r="M71"/>
-      <c s="332" r="N71"/>
-      <c s="333" r="O71"/>
-      <c s="332" r="P71"/>
-      <c s="332" r="Q71"/>
-      <c s="334" r="R71"/>
-      <c s="332" r="S71"/>
-      <c s="332" r="T71"/>
-      <c s="324" r="U71"/>
-      <c s="332" r="V71"/>
-      <c s="332" r="W71"/>
-      <c s="333" r="X71"/>
-      <c s="332" r="Y71"/>
-      <c s="332" r="Z71"/>
-      <c s="333" r="AA71"/>
-      <c s="332" r="AB71"/>
-      <c s="332" r="AC71"/>
-      <c s="333" r="AD71"/>
-      <c s="332" r="AE71"/>
-      <c s="332" r="AF71"/>
-      <c s="333" r="AG71"/>
-      <c s="332" r="AH71"/>
-      <c s="332" r="AI71"/>
-      <c s="334" r="AJ71"/>
-      <c s="332" r="AK71"/>
-      <c s="332" r="AL71"/>
-      <c s="324" r="AM71"/>
-      <c s="332" r="AN71"/>
-      <c s="332" r="AO71"/>
-      <c s="333" r="AP71"/>
-      <c s="332" r="AQ71"/>
-      <c s="332" r="AR71"/>
-      <c s="333" r="AS71"/>
-      <c s="332" r="AT71"/>
-      <c s="332" r="AU71"/>
-      <c s="333" r="AV71"/>
-      <c s="332" r="AW71"/>
-      <c s="332" r="AX71"/>
-      <c s="333" r="AY71"/>
-      <c s="332" r="AZ71"/>
-      <c s="332" r="BA71"/>
-      <c s="334" r="BB71"/>
-      <c s="332" r="BC71"/>
-      <c s="332" r="BD71"/>
-      <c s="324" r="BE71"/>
-      <c s="332" r="BF71"/>
-      <c s="332" r="BG71"/>
-      <c s="333" r="BH71"/>
-      <c s="332" r="BI71"/>
-      <c s="332" r="BJ71"/>
-      <c s="333" r="BK71"/>
-      <c s="332" r="BL71"/>
-      <c s="332" r="BM71"/>
-      <c s="333" r="BN71"/>
-      <c s="332" r="BO71"/>
-      <c s="332" r="BP71"/>
-      <c s="333" r="BQ71"/>
-      <c s="332" r="BR71"/>
-      <c s="332" r="BS71"/>
-      <c s="334" r="BT71"/>
-      <c s="332" r="BU71"/>
-      <c s="332" r="BV71"/>
-      <c s="324" r="BW71"/>
-      <c s="332" r="BX71"/>
-      <c s="332" r="BY71"/>
-      <c s="333" r="BZ71"/>
-      <c s="332" r="CA71"/>
-      <c s="332" r="CB71"/>
-      <c s="333" r="CC71"/>
-      <c s="332" r="CD71"/>
-      <c s="332" r="CE71"/>
-      <c s="333" r="CF71"/>
-      <c s="332" r="CG71"/>
-      <c s="332" r="CH71"/>
-      <c s="333" r="CI71"/>
-      <c s="332" r="CJ71"/>
-      <c s="332" r="CK71"/>
-      <c s="334" r="CL71"/>
-      <c s="332" r="CM71"/>
-      <c s="332" r="CN71"/>
-      <c s="325" r="CO71"/>
-      <c s="332" r="CP71"/>
-      <c s="332" r="CQ71"/>
-      <c s="326" r="CR71"/>
-      <c s="332" r="CS71"/>
-      <c s="332" r="CT71"/>
-      <c s="326" r="CU71"/>
-      <c s="332" r="CV71"/>
-      <c s="332" r="CW71"/>
-      <c s="326" r="CX71"/>
-      <c s="332" r="CY71"/>
-      <c s="332" r="CZ71"/>
-      <c s="326" r="DA71"/>
-      <c s="332" r="DB71"/>
-      <c s="332" r="DC71"/>
-      <c s="326" r="DD71"/>
-      <c s="332" r="DE71"/>
-      <c s="332" r="DF71"/>
-      <c s="335" r="DG71"/>
+    <row r="71" ht="22" customHeight="1">
+      <c s="995" r="A71"/>
+      <c s="996" r="B71"/>
+      <c s="995" r="C71"/>
+      <c s="997" r="D71"/>
+      <c s="998" r="E71"/>
+      <c s="995" r="F71"/>
+      <c s="997" r="G71"/>
+      <c s="998" r="H71"/>
+      <c s="995" r="I71"/>
+      <c s="997" r="J71"/>
+      <c s="998" r="K71"/>
+      <c s="995" r="L71"/>
+      <c s="997" r="M71"/>
+      <c s="998" r="N71"/>
+      <c s="995" r="O71"/>
+      <c s="997" r="P71"/>
+      <c s="998" r="Q71"/>
+      <c s="995" r="R71"/>
+      <c s="999" r="S71"/>
+      <c s="998" r="T71"/>
+      <c s="995" r="U71"/>
+      <c s="997" r="V71"/>
+      <c s="998" r="W71"/>
+      <c s="995" r="X71"/>
+      <c s="997" r="Y71"/>
+      <c s="998" r="Z71"/>
+      <c s="995" r="AA71"/>
+      <c s="997" r="AB71"/>
+      <c s="998" r="AC71"/>
+      <c s="995" r="AD71"/>
+      <c s="997" r="AE71"/>
+      <c s="998" r="AF71"/>
+      <c s="995" r="AG71"/>
+      <c s="997" r="AH71"/>
+      <c s="998" r="AI71"/>
+      <c s="995" r="AJ71"/>
+      <c s="999" r="AK71"/>
+      <c s="998" r="AL71"/>
+      <c s="995" r="AM71"/>
+      <c s="997" r="AN71"/>
+      <c s="998" r="AO71"/>
+      <c s="995" r="AP71"/>
+      <c s="997" r="AQ71"/>
+      <c s="998" r="AR71"/>
+      <c s="995" r="AS71"/>
+      <c s="997" r="AT71"/>
+      <c s="998" r="AU71"/>
+      <c s="995" r="AV71"/>
+      <c s="997" r="AW71"/>
+      <c s="998" r="AX71"/>
+      <c s="995" r="AY71"/>
+      <c s="997" r="AZ71"/>
+      <c s="998" r="BA71"/>
+      <c s="995" r="BB71"/>
+      <c s="999" r="BC71"/>
+      <c s="998" r="BD71"/>
+      <c s="995" r="BE71"/>
+      <c s="997" r="BF71"/>
+      <c s="998" r="BG71"/>
+      <c s="995" r="BH71"/>
+      <c s="997" r="BI71"/>
+      <c s="998" r="BJ71"/>
+      <c s="995" r="BK71"/>
+      <c s="997" r="BL71"/>
+      <c s="998" r="BM71"/>
+      <c s="995" r="BN71"/>
+      <c s="997" r="BO71"/>
+      <c s="998" r="BP71"/>
+      <c s="995" r="BQ71"/>
+      <c s="997" r="BR71"/>
+      <c s="998" r="BS71"/>
+      <c s="995" r="BT71"/>
+      <c s="999" r="BU71"/>
+      <c s="998" r="BV71"/>
+      <c s="995" r="BW71"/>
+      <c s="997" r="BX71"/>
+      <c s="998" r="BY71"/>
+      <c s="995" r="BZ71"/>
+      <c s="997" r="CA71"/>
+      <c s="998" r="CB71"/>
+      <c s="995" r="CC71"/>
+      <c s="997" r="CD71"/>
+      <c s="998" r="CE71"/>
+      <c s="995" r="CF71"/>
+      <c s="997" r="CG71"/>
+      <c s="998" r="CH71"/>
+      <c s="995" r="CI71"/>
+      <c s="997" r="CJ71"/>
+      <c s="998" r="CK71"/>
+      <c s="995" r="CL71"/>
+      <c s="999" r="CM71"/>
+      <c s="998" r="CN71"/>
+      <c s="995" r="CO71"/>
+      <c s="999" r="CP71"/>
+      <c s="998" r="CQ71"/>
+      <c s="995" r="CR71"/>
+      <c s="999" r="CS71"/>
+      <c s="998" r="CT71"/>
+      <c s="995" r="CU71"/>
+      <c s="999" r="CV71"/>
+      <c s="998" r="CW71"/>
+      <c s="995" r="CX71"/>
+      <c s="999" r="CY71"/>
+      <c s="998" r="CZ71"/>
+      <c s="995" r="DA71"/>
+      <c s="999" r="DB71"/>
+      <c s="998" r="DC71"/>
+      <c s="995" r="DD71"/>
+      <c s="999" r="DE71"/>
+      <c s="998" r="DF71"/>
+      <c s="995" r="DG71"/>
     </row>
-    <row r="72" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A72"/>
-      <c s="343" r="B72" t="str">
+    <row r="72" ht="23" customHeight="1">
+      <c s="995" r="A72"/>
+      <c s="1000" r="B72" t="str">
         <v>计算参数</v>
       </c>
-      <c s="331" r="C72"/>
-      <c s="332" r="D72" t="str">
+      <c s="995" r="C72"/>
+      <c s="1001" r="D72" t="str">
         <v>按上方同列的年度、车型填写</v>
       </c>
-      <c s="332" r="E72"/>
-      <c s="333" r="F72"/>
-      <c s="332" r="G72"/>
-      <c s="332" r="H72"/>
-      <c s="333" r="I72"/>
-      <c s="332" r="J72"/>
-      <c s="332" r="K72"/>
-      <c s="333" r="L72"/>
-      <c s="332" r="M72"/>
-      <c s="332" r="N72"/>
-      <c s="333" r="O72"/>
-      <c s="332" r="P72"/>
-      <c s="332" r="Q72"/>
-      <c s="334" r="R72"/>
-      <c s="332" r="S72"/>
-      <c s="332" r="T72"/>
-      <c s="324" r="U72"/>
-      <c s="332" r="V72"/>
-      <c s="332" r="W72"/>
-      <c s="333" r="X72"/>
-      <c s="332" r="Y72"/>
-      <c s="332" r="Z72"/>
-      <c s="333" r="AA72"/>
-      <c s="332" r="AB72"/>
-      <c s="332" r="AC72"/>
-      <c s="333" r="AD72"/>
-      <c s="332" r="AE72"/>
-      <c s="332" r="AF72"/>
-      <c s="333" r="AG72"/>
-      <c s="332" r="AH72"/>
-      <c s="332" r="AI72"/>
-      <c s="334" r="AJ72"/>
-      <c s="332" r="AK72"/>
-      <c s="332" r="AL72"/>
-      <c s="324" r="AM72"/>
-      <c s="332" r="AN72"/>
-      <c s="332" r="AO72"/>
-      <c s="333" r="AP72"/>
-      <c s="332" r="AQ72"/>
-      <c s="332" r="AR72"/>
-      <c s="333" r="AS72"/>
-      <c s="332" r="AT72"/>
-      <c s="332" r="AU72"/>
-      <c s="333" r="AV72"/>
-      <c s="332" r="AW72"/>
-      <c s="332" r="AX72"/>
-      <c s="333" r="AY72"/>
-      <c s="332" r="AZ72"/>
-      <c s="332" r="BA72"/>
-      <c s="334" r="BB72"/>
-      <c s="332" r="BC72"/>
-      <c s="332" r="BD72"/>
-      <c s="324" r="BE72"/>
-      <c s="332" r="BF72"/>
-      <c s="332" r="BG72"/>
-      <c s="333" r="BH72"/>
-      <c s="332" r="BI72"/>
-      <c s="332" r="BJ72"/>
-      <c s="333" r="BK72"/>
-      <c s="332" r="BL72"/>
-      <c s="332" r="BM72"/>
-      <c s="333" r="BN72"/>
-      <c s="332" r="BO72"/>
-      <c s="332" r="BP72"/>
-      <c s="333" r="BQ72"/>
-      <c s="332" r="BR72"/>
-      <c s="332" r="BS72"/>
-      <c s="334" r="BT72"/>
-      <c s="332" r="BU72"/>
-      <c s="332" r="BV72"/>
-      <c s="324" r="BW72"/>
-      <c s="332" r="BX72"/>
-      <c s="332" r="BY72"/>
-      <c s="333" r="BZ72"/>
-      <c s="332" r="CA72"/>
-      <c s="332" r="CB72"/>
-      <c s="333" r="CC72"/>
-      <c s="332" r="CD72"/>
-      <c s="332" r="CE72"/>
-      <c s="333" r="CF72"/>
-      <c s="332" r="CG72"/>
-      <c s="332" r="CH72"/>
-      <c s="333" r="CI72"/>
-      <c s="332" r="CJ72"/>
-      <c s="332" r="CK72"/>
-      <c s="334" r="CL72"/>
-      <c s="332" r="CM72"/>
-      <c s="332" r="CN72"/>
-      <c s="325" r="CO72"/>
-      <c s="332" r="CP72"/>
-      <c s="332" r="CQ72"/>
-      <c s="326" r="CR72"/>
-      <c s="332" r="CS72"/>
-      <c s="332" r="CT72"/>
-      <c s="326" r="CU72"/>
-      <c s="332" r="CV72"/>
-      <c s="332" r="CW72"/>
-      <c s="326" r="CX72"/>
-      <c s="332" r="CY72"/>
-      <c s="332" r="CZ72"/>
-      <c s="326" r="DA72"/>
-      <c s="332" r="DB72"/>
-      <c s="332" r="DC72"/>
-      <c s="326" r="DD72"/>
-      <c s="332" r="DE72"/>
-      <c s="332" r="DF72"/>
-      <c s="335" r="DG72"/>
+      <c s="1001" r="E72"/>
+      <c s="1001" r="F72"/>
+      <c s="1001" r="G72"/>
+      <c s="1001" r="H72"/>
+      <c s="1001" r="I72"/>
+      <c s="1001" r="J72"/>
+      <c s="1001" r="K72"/>
+      <c s="1001" r="L72"/>
+      <c s="1001" r="M72"/>
+      <c s="1001" r="N72"/>
+      <c s="1001" r="O72"/>
+      <c s="1001" r="P72"/>
+      <c s="1001" r="Q72"/>
+      <c s="1001" r="R72"/>
+      <c s="1001" r="S72"/>
+      <c s="1001" r="T72"/>
+      <c s="995" r="U72"/>
+      <c s="995" r="V72"/>
+      <c s="995" r="W72"/>
+      <c s="995" r="X72"/>
+      <c s="995" r="Y72"/>
+      <c s="995" r="Z72"/>
+      <c s="995" r="AA72"/>
+      <c s="995" r="AB72"/>
+      <c s="995" r="AC72"/>
+      <c s="995" r="AD72"/>
+      <c s="995" r="AE72"/>
+      <c s="995" r="AF72"/>
+      <c s="995" r="AG72"/>
+      <c s="995" r="AH72"/>
+      <c s="995" r="AI72"/>
+      <c s="995" r="AJ72"/>
+      <c s="995" r="AK72"/>
+      <c s="995" r="AL72"/>
+      <c s="995" r="AM72"/>
+      <c s="995" r="AN72"/>
+      <c s="995" r="AO72"/>
+      <c s="995" r="AP72"/>
+      <c s="995" r="AQ72"/>
+      <c s="995" r="AR72"/>
+      <c s="995" r="AS72"/>
+      <c s="995" r="AT72"/>
+      <c s="995" r="AU72"/>
+      <c s="995" r="AV72"/>
+      <c s="995" r="AW72"/>
+      <c s="995" r="AX72"/>
+      <c s="995" r="AY72"/>
+      <c s="995" r="AZ72"/>
+      <c s="995" r="BA72"/>
+      <c s="995" r="BB72"/>
+      <c s="995" r="BC72"/>
+      <c s="995" r="BD72"/>
+      <c s="995" r="BE72"/>
+      <c s="995" r="BF72"/>
+      <c s="995" r="BG72"/>
+      <c s="995" r="BH72"/>
+      <c s="995" r="BI72"/>
+      <c s="995" r="BJ72"/>
+      <c s="995" r="BK72"/>
+      <c s="995" r="BL72"/>
+      <c s="995" r="BM72"/>
+      <c s="995" r="BN72"/>
+      <c s="995" r="BO72"/>
+      <c s="995" r="BP72"/>
+      <c s="995" r="BQ72"/>
+      <c s="995" r="BR72"/>
+      <c s="995" r="BS72"/>
+      <c s="995" r="BT72"/>
+      <c s="995" r="BU72"/>
+      <c s="995" r="BV72"/>
+      <c s="995" r="BW72"/>
+      <c s="995" r="BX72"/>
+      <c s="995" r="BY72"/>
+      <c s="995" r="BZ72"/>
+      <c s="995" r="CA72"/>
+      <c s="995" r="CB72"/>
+      <c s="995" r="CC72"/>
+      <c s="995" r="CD72"/>
+      <c s="995" r="CE72"/>
+      <c s="995" r="CF72"/>
+      <c s="995" r="CG72"/>
+      <c s="995" r="CH72"/>
+      <c s="995" r="CI72"/>
+      <c s="995" r="CJ72"/>
+      <c s="995" r="CK72"/>
+      <c s="995" r="CL72"/>
+      <c s="995" r="CM72"/>
+      <c s="995" r="CN72"/>
+      <c s="995" r="CO72"/>
+      <c s="995" r="CP72"/>
+      <c s="995" r="CQ72"/>
+      <c s="995" r="CR72"/>
+      <c s="995" r="CS72"/>
+      <c s="995" r="CT72"/>
+      <c s="995" r="CU72"/>
+      <c s="995" r="CV72"/>
+      <c s="995" r="CW72"/>
+      <c s="995" r="CX72"/>
+      <c s="995" r="CY72"/>
+      <c s="995" r="CZ72"/>
+      <c s="995" r="DA72"/>
+      <c s="995" r="DB72"/>
+      <c s="995" r="DC72"/>
+      <c s="995" r="DD72"/>
+      <c s="995" r="DE72"/>
+      <c s="995" r="DF72"/>
+      <c s="995" r="DG72"/>
     </row>
-    <row r="73" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A73"/>
-      <c s="322" r="B73" t="str">
+    <row r="73" ht="23" customHeight="1">
+      <c s="995" r="A73"/>
+      <c s="1002" r="B73" t="str">
         <v>增值税率</v>
       </c>
-      <c s="331" r="C73"/>
-      <c s="361" r="D73"/>
-      <c s="332" r="E73"/>
-      <c s="333" r="F73"/>
-      <c s="361" r="G73"/>
-      <c s="332" r="H73"/>
-      <c s="333" r="I73"/>
-      <c s="361" r="J73"/>
-      <c s="332" r="K73"/>
-      <c s="333" r="L73"/>
-      <c s="361" r="M73"/>
-      <c s="332" r="N73"/>
-      <c s="333" r="O73"/>
-      <c s="361" r="P73"/>
-      <c s="332" r="Q73"/>
-      <c s="334" r="R73"/>
-      <c s="332" r="S73"/>
-      <c s="332" r="T73"/>
-      <c s="324" r="U73"/>
-      <c s="361" r="V73"/>
-      <c s="332" r="W73"/>
-      <c s="333" r="X73"/>
-      <c s="361" r="Y73"/>
-      <c s="332" r="Z73"/>
-      <c s="333" r="AA73"/>
-      <c s="361" r="AB73"/>
-      <c s="332" r="AC73"/>
-      <c s="333" r="AD73"/>
-      <c s="361" r="AE73"/>
-      <c s="332" r="AF73"/>
-      <c s="333" r="AG73"/>
-      <c s="361" r="AH73"/>
-      <c s="332" r="AI73"/>
-      <c s="334" r="AJ73"/>
-      <c s="332" r="AK73"/>
-      <c s="332" r="AL73"/>
-      <c s="324" r="AM73"/>
-      <c s="361" r="AN73"/>
-      <c s="332" r="AO73"/>
-      <c s="333" r="AP73"/>
-      <c s="361" r="AQ73"/>
-      <c s="332" r="AR73"/>
-      <c s="333" r="AS73"/>
-      <c s="361" r="AT73"/>
-      <c s="332" r="AU73"/>
-      <c s="333" r="AV73"/>
-      <c s="361" r="AW73"/>
-      <c s="332" r="AX73"/>
-      <c s="333" r="AY73"/>
-      <c s="361" r="AZ73"/>
-      <c s="332" r="BA73"/>
-      <c s="334" r="BB73"/>
-      <c s="332" r="BC73"/>
-      <c s="332" r="BD73"/>
-      <c s="324" r="BE73"/>
-      <c s="361" r="BF73"/>
-      <c s="332" r="BG73"/>
-      <c s="333" r="BH73"/>
-      <c s="361" r="BI73"/>
-      <c s="332" r="BJ73"/>
-      <c s="333" r="BK73"/>
-      <c s="361" r="BL73"/>
-      <c s="332" r="BM73"/>
-      <c s="333" r="BN73"/>
-      <c s="361" r="BO73"/>
-      <c s="332" r="BP73"/>
-      <c s="333" r="BQ73"/>
-      <c s="361" r="BR73"/>
-      <c s="332" r="BS73"/>
-      <c s="334" r="BT73"/>
-      <c s="332" r="BU73"/>
-      <c s="332" r="BV73"/>
-      <c s="324" r="BW73"/>
-      <c s="361" r="BX73"/>
-      <c s="332" r="BY73"/>
-      <c s="333" r="BZ73"/>
-      <c s="361" r="CA73"/>
-      <c s="332" r="CB73"/>
-      <c s="333" r="CC73"/>
-      <c s="361" r="CD73"/>
-      <c s="332" r="CE73"/>
-      <c s="333" r="CF73"/>
-      <c s="361" r="CG73"/>
-      <c s="332" r="CH73"/>
-      <c s="333" r="CI73"/>
-      <c s="361" r="CJ73"/>
-      <c s="332" r="CK73"/>
-      <c s="334" r="CL73"/>
-      <c s="332" r="CM73"/>
-      <c s="332" r="CN73"/>
-      <c s="325" r="CO73"/>
-      <c s="332" r="CP73"/>
-      <c s="332" r="CQ73"/>
-      <c s="326" r="CR73"/>
-      <c s="332" r="CS73"/>
-      <c s="332" r="CT73"/>
-      <c s="326" r="CU73"/>
-      <c s="332" r="CV73"/>
-      <c s="332" r="CW73"/>
-      <c s="326" r="CX73"/>
-      <c s="332" r="CY73"/>
-      <c s="332" r="CZ73"/>
-      <c s="326" r="DA73"/>
-      <c s="332" r="DB73"/>
-      <c s="332" r="DC73"/>
-      <c s="326" r="DD73"/>
-      <c s="332" r="DE73"/>
-      <c s="332" r="DF73"/>
-      <c s="335" r="DG73"/>
+      <c s="995" r="C73"/>
+      <c s="1003" r="D73"/>
+      <c s="998" r="E73"/>
+      <c s="995" r="F73"/>
+      <c s="1003" r="G73"/>
+      <c s="998" r="H73"/>
+      <c s="995" r="I73"/>
+      <c s="1003" r="J73"/>
+      <c s="998" r="K73"/>
+      <c s="995" r="L73"/>
+      <c s="1003" r="M73"/>
+      <c s="998" r="N73"/>
+      <c s="995" r="O73"/>
+      <c s="1003" r="P73"/>
+      <c s="998" r="Q73"/>
+      <c s="995" r="R73"/>
+      <c s="1004" r="S73"/>
+      <c s="998" r="T73"/>
+      <c s="995" r="U73"/>
+      <c s="1003" r="V73"/>
+      <c s="998" r="W73"/>
+      <c s="995" r="X73"/>
+      <c s="1003" r="Y73"/>
+      <c s="998" r="Z73"/>
+      <c s="995" r="AA73"/>
+      <c s="1003" r="AB73"/>
+      <c s="998" r="AC73"/>
+      <c s="995" r="AD73"/>
+      <c s="1003" r="AE73"/>
+      <c s="998" r="AF73"/>
+      <c s="995" r="AG73"/>
+      <c s="1003" r="AH73"/>
+      <c s="998" r="AI73"/>
+      <c s="995" r="AJ73"/>
+      <c s="1004" r="AK73"/>
+      <c s="998" r="AL73"/>
+      <c s="995" r="AM73"/>
+      <c s="1003" r="AN73"/>
+      <c s="998" r="AO73"/>
+      <c s="995" r="AP73"/>
+      <c s="1003" r="AQ73"/>
+      <c s="998" r="AR73"/>
+      <c s="995" r="AS73"/>
+      <c s="1003" r="AT73"/>
+      <c s="998" r="AU73"/>
+      <c s="995" r="AV73"/>
+      <c s="1003" r="AW73"/>
+      <c s="998" r="AX73"/>
+      <c s="995" r="AY73"/>
+      <c s="1003" r="AZ73"/>
+      <c s="998" r="BA73"/>
+      <c s="995" r="BB73"/>
+      <c s="1004" r="BC73"/>
+      <c s="998" r="BD73"/>
+      <c s="995" r="BE73"/>
+      <c s="1003" r="BF73"/>
+      <c s="998" r="BG73"/>
+      <c s="995" r="BH73"/>
+      <c s="1003" r="BI73"/>
+      <c s="998" r="BJ73"/>
+      <c s="995" r="BK73"/>
+      <c s="1003" r="BL73"/>
+      <c s="998" r="BM73"/>
+      <c s="995" r="BN73"/>
+      <c s="1003" r="BO73"/>
+      <c s="998" r="BP73"/>
+      <c s="995" r="BQ73"/>
+      <c s="1003" r="BR73"/>
+      <c s="998" r="BS73"/>
+      <c s="995" r="BT73"/>
+      <c s="1004" r="BU73"/>
+      <c s="998" r="BV73"/>
+      <c s="995" r="BW73"/>
+      <c s="1003" r="BX73"/>
+      <c s="998" r="BY73"/>
+      <c s="995" r="BZ73"/>
+      <c s="1003" r="CA73"/>
+      <c s="998" r="CB73"/>
+      <c s="995" r="CC73"/>
+      <c s="1003" r="CD73"/>
+      <c s="998" r="CE73"/>
+      <c s="995" r="CF73"/>
+      <c s="1003" r="CG73"/>
+      <c s="998" r="CH73"/>
+      <c s="995" r="CI73"/>
+      <c s="1003" r="CJ73"/>
+      <c s="998" r="CK73"/>
+      <c s="995" r="CL73"/>
+      <c s="1004" r="CM73"/>
+      <c s="998" r="CN73"/>
+      <c s="995" r="CO73"/>
+      <c s="1004" r="CP73"/>
+      <c s="998" r="CQ73"/>
+      <c s="995" r="CR73"/>
+      <c s="1004" r="CS73"/>
+      <c s="998" r="CT73"/>
+      <c s="995" r="CU73"/>
+      <c s="1004" r="CV73"/>
+      <c s="998" r="CW73"/>
+      <c s="995" r="CX73"/>
+      <c s="1004" r="CY73"/>
+      <c s="998" r="CZ73"/>
+      <c s="995" r="DA73"/>
+      <c s="1004" r="DB73"/>
+      <c s="998" r="DC73"/>
+      <c s="995" r="DD73"/>
+      <c s="1004" r="DE73"/>
+      <c s="998" r="DF73"/>
+      <c s="995" r="DG73"/>
     </row>
-    <row r="74" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A74"/>
-      <c s="322" r="B74" t="str">
+    <row r="74" ht="23" customHeight="1">
+      <c s="995" r="A74"/>
+      <c s="1002" r="B74" t="str">
         <v>消费税率</v>
       </c>
-      <c s="331" r="C74"/>
-      <c s="361" r="D74"/>
-      <c s="332" r="E74"/>
-      <c s="333" r="F74"/>
-      <c s="361" r="G74"/>
-      <c s="332" r="H74"/>
-      <c s="333" r="I74"/>
-      <c s="361" r="J74"/>
-      <c s="332" r="K74"/>
-      <c s="333" r="L74"/>
-      <c s="361" r="M74"/>
-      <c s="332" r="N74"/>
-      <c s="333" r="O74"/>
-      <c s="361" r="P74"/>
-      <c s="332" r="Q74"/>
-      <c s="334" r="R74"/>
-      <c s="332" r="S74"/>
-      <c s="332" r="T74"/>
-      <c s="324" r="U74"/>
-      <c s="361" r="V74"/>
-      <c s="332" r="W74"/>
-      <c s="333" r="X74"/>
-      <c s="361" r="Y74"/>
-      <c s="332" r="Z74"/>
-      <c s="333" r="AA74"/>
-      <c s="361" r="AB74"/>
-      <c s="332" r="AC74"/>
-      <c s="333" r="AD74"/>
-      <c s="361" r="AE74"/>
-      <c s="332" r="AF74"/>
-      <c s="333" r="AG74"/>
-      <c s="361" r="AH74"/>
-      <c s="332" r="AI74"/>
-      <c s="334" r="AJ74"/>
-      <c s="332" r="AK74"/>
-      <c s="332" r="AL74"/>
-      <c s="324" r="AM74"/>
-      <c s="361" r="AN74"/>
-      <c s="332" r="AO74"/>
-      <c s="333" r="AP74"/>
-      <c s="361" r="AQ74"/>
-      <c s="332" r="AR74"/>
-      <c s="333" r="AS74"/>
-      <c s="361" r="AT74"/>
-      <c s="332" r="AU74"/>
-      <c s="333" r="AV74"/>
-      <c s="361" r="AW74"/>
-      <c s="332" r="AX74"/>
-      <c s="333" r="AY74"/>
-      <c s="361" r="AZ74"/>
-      <c s="332" r="BA74"/>
-      <c s="334" r="BB74"/>
-      <c s="332" r="BC74"/>
-      <c s="332" r="BD74"/>
-      <c s="324" r="BE74"/>
-      <c s="361" r="BF74"/>
-      <c s="332" r="BG74"/>
-      <c s="333" r="BH74"/>
-      <c s="361" r="BI74"/>
-      <c s="332" r="BJ74"/>
-      <c s="333" r="BK74"/>
-      <c s="361" r="BL74"/>
-      <c s="332" r="BM74"/>
-      <c s="333" r="BN74"/>
-      <c s="361" r="BO74"/>
-      <c s="332" r="BP74"/>
-      <c s="333" r="BQ74"/>
-      <c s="361" r="BR74"/>
-      <c s="332" r="BS74"/>
-      <c s="334" r="BT74"/>
-      <c s="332" r="BU74"/>
-      <c s="332" r="BV74"/>
-      <c s="324" r="BW74"/>
-      <c s="361" r="BX74"/>
-      <c s="332" r="BY74"/>
-      <c s="333" r="BZ74"/>
-      <c s="361" r="CA74"/>
-      <c s="332" r="CB74"/>
-      <c s="333" r="CC74"/>
-      <c s="361" r="CD74"/>
-      <c s="332" r="CE74"/>
-      <c s="333" r="CF74"/>
-      <c s="361" r="CG74"/>
-      <c s="332" r="CH74"/>
-      <c s="333" r="CI74"/>
-      <c s="361" r="CJ74"/>
-      <c s="332" r="CK74"/>
-      <c s="334" r="CL74"/>
-      <c s="332" r="CM74"/>
-      <c s="332" r="CN74"/>
-      <c s="325" r="CO74"/>
-      <c s="332" r="CP74"/>
-      <c s="332" r="CQ74"/>
-      <c s="326" r="CR74"/>
-      <c s="332" r="CS74"/>
-      <c s="332" r="CT74"/>
-      <c s="326" r="CU74"/>
-      <c s="332" r="CV74"/>
-      <c s="332" r="CW74"/>
-      <c s="326" r="CX74"/>
-      <c s="332" r="CY74"/>
-      <c s="332" r="CZ74"/>
-      <c s="326" r="DA74"/>
-      <c s="332" r="DB74"/>
-      <c s="332" r="DC74"/>
-      <c s="326" r="DD74"/>
-      <c s="332" r="DE74"/>
-      <c s="332" r="DF74"/>
-      <c s="335" r="DG74"/>
+      <c s="995" r="C74"/>
+      <c s="1003" r="D74"/>
+      <c s="998" r="E74"/>
+      <c s="995" r="F74"/>
+      <c s="1003" r="G74"/>
+      <c s="998" r="H74"/>
+      <c s="995" r="I74"/>
+      <c s="1003" r="J74"/>
+      <c s="998" r="K74"/>
+      <c s="995" r="L74"/>
+      <c s="1003" r="M74"/>
+      <c s="998" r="N74"/>
+      <c s="995" r="O74"/>
+      <c s="1003" r="P74"/>
+      <c s="998" r="Q74"/>
+      <c s="995" r="R74"/>
+      <c s="1004" r="S74"/>
+      <c s="998" r="T74"/>
+      <c s="995" r="U74"/>
+      <c s="1003" r="V74"/>
+      <c s="998" r="W74"/>
+      <c s="995" r="X74"/>
+      <c s="1003" r="Y74"/>
+      <c s="998" r="Z74"/>
+      <c s="995" r="AA74"/>
+      <c s="1003" r="AB74"/>
+      <c s="998" r="AC74"/>
+      <c s="995" r="AD74"/>
+      <c s="1003" r="AE74"/>
+      <c s="998" r="AF74"/>
+      <c s="995" r="AG74"/>
+      <c s="1003" r="AH74"/>
+      <c s="998" r="AI74"/>
+      <c s="995" r="AJ74"/>
+      <c s="1004" r="AK74"/>
+      <c s="998" r="AL74"/>
+      <c s="995" r="AM74"/>
+      <c s="1003" r="AN74"/>
+      <c s="998" r="AO74"/>
+      <c s="995" r="AP74"/>
+      <c s="1003" r="AQ74"/>
+      <c s="998" r="AR74"/>
+      <c s="995" r="AS74"/>
+      <c s="1003" r="AT74"/>
+      <c s="998" r="AU74"/>
+      <c s="995" r="AV74"/>
+      <c s="1003" r="AW74"/>
+      <c s="998" r="AX74"/>
+      <c s="995" r="AY74"/>
+      <c s="1003" r="AZ74"/>
+      <c s="998" r="BA74"/>
+      <c s="995" r="BB74"/>
+      <c s="1004" r="BC74"/>
+      <c s="998" r="BD74"/>
+      <c s="995" r="BE74"/>
+      <c s="1003" r="BF74"/>
+      <c s="998" r="BG74"/>
+      <c s="995" r="BH74"/>
+      <c s="1003" r="BI74"/>
+      <c s="998" r="BJ74"/>
+      <c s="995" r="BK74"/>
+      <c s="1003" r="BL74"/>
+      <c s="998" r="BM74"/>
+      <c s="995" r="BN74"/>
+      <c s="1003" r="BO74"/>
+      <c s="998" r="BP74"/>
+      <c s="995" r="BQ74"/>
+      <c s="1003" r="BR74"/>
+      <c s="998" r="BS74"/>
+      <c s="995" r="BT74"/>
+      <c s="1004" r="BU74"/>
+      <c s="998" r="BV74"/>
+      <c s="995" r="BW74"/>
+      <c s="1003" r="BX74"/>
+      <c s="998" r="BY74"/>
+      <c s="995" r="BZ74"/>
+      <c s="1003" r="CA74"/>
+      <c s="998" r="CB74"/>
+      <c s="995" r="CC74"/>
+      <c s="1003" r="CD74"/>
+      <c s="998" r="CE74"/>
+      <c s="995" r="CF74"/>
+      <c s="1003" r="CG74"/>
+      <c s="998" r="CH74"/>
+      <c s="995" r="CI74"/>
+      <c s="1003" r="CJ74"/>
+      <c s="998" r="CK74"/>
+      <c s="995" r="CL74"/>
+      <c s="1004" r="CM74"/>
+      <c s="998" r="CN74"/>
+      <c s="995" r="CO74"/>
+      <c s="1004" r="CP74"/>
+      <c s="998" r="CQ74"/>
+      <c s="995" r="CR74"/>
+      <c s="1004" r="CS74"/>
+      <c s="998" r="CT74"/>
+      <c s="995" r="CU74"/>
+      <c s="1004" r="CV74"/>
+      <c s="998" r="CW74"/>
+      <c s="995" r="CX74"/>
+      <c s="1004" r="CY74"/>
+      <c s="998" r="CZ74"/>
+      <c s="995" r="DA74"/>
+      <c s="1004" r="DB74"/>
+      <c s="998" r="DC74"/>
+      <c s="995" r="DD74"/>
+      <c s="1004" r="DE74"/>
+      <c s="998" r="DF74"/>
+      <c s="995" r="DG74"/>
     </row>
-    <row r="75" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A75"/>
-      <c s="322" r="B75" t="str">
+    <row r="75" ht="23" customHeight="1">
+      <c s="995" r="A75"/>
+      <c s="1002" r="B75" t="str">
         <v>城建税及教育附加综合税率</v>
       </c>
-      <c s="331" r="C75"/>
-      <c s="361" r="D75"/>
-      <c s="332" r="E75"/>
-      <c s="333" r="F75"/>
-      <c s="361" r="G75"/>
-      <c s="332" r="H75"/>
-      <c s="333" r="I75"/>
-      <c s="361" r="J75"/>
-      <c s="332" r="K75"/>
-      <c s="333" r="L75"/>
-      <c s="361" r="M75"/>
-      <c s="332" r="N75"/>
-      <c s="333" r="O75"/>
-      <c s="361" r="P75"/>
-      <c s="332" r="Q75"/>
-      <c s="334" r="R75"/>
-      <c s="332" r="S75"/>
-      <c s="332" r="T75"/>
-      <c s="324" r="U75"/>
-      <c s="361" r="V75"/>
-      <c s="332" r="W75"/>
-      <c s="333" r="X75"/>
-      <c s="361" r="Y75"/>
-      <c s="332" r="Z75"/>
-      <c s="333" r="AA75"/>
-      <c s="361" r="AB75"/>
-      <c s="332" r="AC75"/>
-      <c s="333" r="AD75"/>
-      <c s="361" r="AE75"/>
-      <c s="332" r="AF75"/>
-      <c s="333" r="AG75"/>
-      <c s="361" r="AH75"/>
-      <c s="332" r="AI75"/>
-      <c s="334" r="AJ75"/>
-      <c s="332" r="AK75"/>
-      <c s="332" r="AL75"/>
-      <c s="324" r="AM75"/>
-      <c s="361" r="AN75"/>
-      <c s="332" r="AO75"/>
-      <c s="333" r="AP75"/>
-      <c s="361" r="AQ75"/>
-      <c s="332" r="AR75"/>
-      <c s="333" r="AS75"/>
-      <c s="361" r="AT75"/>
-      <c s="332" r="AU75"/>
-      <c s="333" r="AV75"/>
-      <c s="361" r="AW75"/>
-      <c s="332" r="AX75"/>
-      <c s="333" r="AY75"/>
-      <c s="361" r="AZ75"/>
-      <c s="332" r="BA75"/>
-      <c s="334" r="BB75"/>
-      <c s="332" r="BC75"/>
-      <c s="332" r="BD75"/>
-      <c s="324" r="BE75"/>
-      <c s="361" r="BF75"/>
-      <c s="332" r="BG75"/>
-      <c s="333" r="BH75"/>
-      <c s="361" r="BI75"/>
-      <c s="332" r="BJ75"/>
-      <c s="333" r="BK75"/>
-      <c s="361" r="BL75"/>
-      <c s="332" r="BM75"/>
-      <c s="333" r="BN75"/>
-      <c s="361" r="BO75"/>
-      <c s="332" r="BP75"/>
-      <c s="333" r="BQ75"/>
-      <c s="361" r="BR75"/>
-      <c s="332" r="BS75"/>
-      <c s="334" r="BT75"/>
-      <c s="332" r="BU75"/>
-      <c s="332" r="BV75"/>
-      <c s="324" r="BW75"/>
-      <c s="361" r="BX75"/>
-      <c s="332" r="BY75"/>
-      <c s="333" r="BZ75"/>
-      <c s="361" r="CA75"/>
-      <c s="332" r="CB75"/>
-      <c s="333" r="CC75"/>
-      <c s="361" r="CD75"/>
-      <c s="332" r="CE75"/>
-      <c s="333" r="CF75"/>
-      <c s="361" r="CG75"/>
-      <c s="332" r="CH75"/>
-      <c s="333" r="CI75"/>
-      <c s="361" r="CJ75"/>
-      <c s="332" r="CK75"/>
-      <c s="334" r="CL75"/>
-      <c s="332" r="CM75"/>
-      <c s="332" r="CN75"/>
-      <c s="325" r="CO75"/>
-      <c s="332" r="CP75"/>
-      <c s="332" r="CQ75"/>
-      <c s="326" r="CR75"/>
-      <c s="332" r="CS75"/>
-      <c s="332" r="CT75"/>
-      <c s="326" r="CU75"/>
-      <c s="332" r="CV75"/>
-      <c s="332" r="CW75"/>
-      <c s="326" r="CX75"/>
-      <c s="332" r="CY75"/>
-      <c s="332" r="CZ75"/>
-      <c s="326" r="DA75"/>
-      <c s="332" r="DB75"/>
-      <c s="332" r="DC75"/>
-      <c s="326" r="DD75"/>
-      <c s="332" r="DE75"/>
-      <c s="332" r="DF75"/>
-      <c s="335" r="DG75"/>
+      <c s="995" r="C75"/>
+      <c s="1003" r="D75"/>
+      <c s="998" r="E75"/>
+      <c s="995" r="F75"/>
+      <c s="1003" r="G75"/>
+      <c s="998" r="H75"/>
+      <c s="995" r="I75"/>
+      <c s="1003" r="J75"/>
+      <c s="998" r="K75"/>
+      <c s="995" r="L75"/>
+      <c s="1003" r="M75"/>
+      <c s="998" r="N75"/>
+      <c s="995" r="O75"/>
+      <c s="1003" r="P75"/>
+      <c s="998" r="Q75"/>
+      <c s="995" r="R75"/>
+      <c s="1004" r="S75"/>
+      <c s="998" r="T75"/>
+      <c s="995" r="U75"/>
+      <c s="1003" r="V75"/>
+      <c s="998" r="W75"/>
+      <c s="995" r="X75"/>
+      <c s="1003" r="Y75"/>
+      <c s="998" r="Z75"/>
+      <c s="995" r="AA75"/>
+      <c s="1003" r="AB75"/>
+      <c s="998" r="AC75"/>
+      <c s="995" r="AD75"/>
+      <c s="1003" r="AE75"/>
+      <c s="998" r="AF75"/>
+      <c s="995" r="AG75"/>
+      <c s="1003" r="AH75"/>
+      <c s="998" r="AI75"/>
+      <c s="995" r="AJ75"/>
+      <c s="1004" r="AK75"/>
+      <c s="998" r="AL75"/>
+      <c s="995" r="AM75"/>
+      <c s="1003" r="AN75"/>
+      <c s="998" r="AO75"/>
+      <c s="995" r="AP75"/>
+      <c s="1003" r="AQ75"/>
+      <c s="998" r="AR75"/>
+      <c s="995" r="AS75"/>
+      <c s="1003" r="AT75"/>
+      <c s="998" r="AU75"/>
+      <c s="995" r="AV75"/>
+      <c s="1003" r="AW75"/>
+      <c s="998" r="AX75"/>
+      <c s="995" r="AY75"/>
+      <c s="1003" r="AZ75"/>
+      <c s="998" r="BA75"/>
+      <c s="995" r="BB75"/>
+      <c s="1004" r="BC75"/>
+      <c s="998" r="BD75"/>
+      <c s="995" r="BE75"/>
+      <c s="1003" r="BF75"/>
+      <c s="998" r="BG75"/>
+      <c s="995" r="BH75"/>
+      <c s="1003" r="BI75"/>
+      <c s="998" r="BJ75"/>
+      <c s="995" r="BK75"/>
+      <c s="1003" r="BL75"/>
+      <c s="998" r="BM75"/>
+      <c s="995" r="BN75"/>
+      <c s="1003" r="BO75"/>
+      <c s="998" r="BP75"/>
+      <c s="995" r="BQ75"/>
+      <c s="1003" r="BR75"/>
+      <c s="998" r="BS75"/>
+      <c s="995" r="BT75"/>
+      <c s="1004" r="BU75"/>
+      <c s="998" r="BV75"/>
+      <c s="995" r="BW75"/>
+      <c s="1003" r="BX75"/>
+      <c s="998" r="BY75"/>
+      <c s="995" r="BZ75"/>
+      <c s="1003" r="CA75"/>
+      <c s="998" r="CB75"/>
+      <c s="995" r="CC75"/>
+      <c s="1003" r="CD75"/>
+      <c s="998" r="CE75"/>
+      <c s="995" r="CF75"/>
+      <c s="1003" r="CG75"/>
+      <c s="998" r="CH75"/>
+      <c s="995" r="CI75"/>
+      <c s="1003" r="CJ75"/>
+      <c s="998" r="CK75"/>
+      <c s="995" r="CL75"/>
+      <c s="1004" r="CM75"/>
+      <c s="998" r="CN75"/>
+      <c s="995" r="CO75"/>
+      <c s="1004" r="CP75"/>
+      <c s="998" r="CQ75"/>
+      <c s="995" r="CR75"/>
+      <c s="1004" r="CS75"/>
+      <c s="998" r="CT75"/>
+      <c s="995" r="CU75"/>
+      <c s="1004" r="CV75"/>
+      <c s="998" r="CW75"/>
+      <c s="995" r="CX75"/>
+      <c s="1004" r="CY75"/>
+      <c s="998" r="CZ75"/>
+      <c s="995" r="DA75"/>
+      <c s="1004" r="DB75"/>
+      <c s="998" r="DC75"/>
+      <c s="995" r="DD75"/>
+      <c s="1004" r="DE75"/>
+      <c s="998" r="DF75"/>
+      <c s="995" r="DG75"/>
     </row>
-    <row r="76" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A76"/>
-      <c s="322" r="B76" t="str">
+    <row r="76" ht="23" customHeight="1">
+      <c s="995" r="A76"/>
+      <c s="1002" r="B76" t="str">
         <v>关税计税基数（元/台）</v>
       </c>
-      <c s="331" r="C76"/>
-      <c s="393" r="D76"/>
-      <c s="332" r="E76"/>
-      <c s="333" r="F76"/>
-      <c s="393" r="G76"/>
-      <c s="332" r="H76"/>
-      <c s="333" r="I76"/>
-      <c s="393" r="J76"/>
-      <c s="332" r="K76"/>
-      <c s="333" r="L76"/>
-      <c s="393" r="M76"/>
-      <c s="332" r="N76"/>
-      <c s="333" r="O76"/>
-      <c s="393" r="P76"/>
-      <c s="332" r="Q76"/>
-      <c s="334" r="R76"/>
-      <c s="332" r="S76"/>
-      <c s="332" r="T76"/>
-      <c s="324" r="U76"/>
-      <c s="393" r="V76"/>
-      <c s="332" r="W76"/>
-      <c s="333" r="X76"/>
-      <c s="393" r="Y76"/>
-      <c s="332" r="Z76"/>
-      <c s="333" r="AA76"/>
-      <c s="393" r="AB76"/>
-      <c s="332" r="AC76"/>
-      <c s="333" r="AD76"/>
-      <c s="393" r="AE76"/>
-      <c s="332" r="AF76"/>
-      <c s="333" r="AG76"/>
-      <c s="393" r="AH76"/>
-      <c s="332" r="AI76"/>
-      <c s="334" r="AJ76"/>
-      <c s="332" r="AK76"/>
-      <c s="332" r="AL76"/>
-      <c s="324" r="AM76"/>
-      <c s="393" r="AN76"/>
-      <c s="332" r="AO76"/>
-      <c s="333" r="AP76"/>
-      <c s="393" r="AQ76"/>
-      <c s="332" r="AR76"/>
-      <c s="333" r="AS76"/>
-      <c s="393" r="AT76"/>
-      <c s="332" r="AU76"/>
-      <c s="333" r="AV76"/>
-      <c s="393" r="AW76"/>
-      <c s="332" r="AX76"/>
-      <c s="333" r="AY76"/>
-      <c s="393" r="AZ76"/>
-      <c s="332" r="BA76"/>
-      <c s="334" r="BB76"/>
-      <c s="332" r="BC76"/>
-      <c s="332" r="BD76"/>
-      <c s="324" r="BE76"/>
-      <c s="393" r="BF76"/>
-      <c s="332" r="BG76"/>
-      <c s="333" r="BH76"/>
-      <c s="393" r="BI76"/>
-      <c s="332" r="BJ76"/>
-      <c s="333" r="BK76"/>
-      <c s="393" r="BL76"/>
-      <c s="332" r="BM76"/>
-      <c s="333" r="BN76"/>
-      <c s="393" r="BO76"/>
-      <c s="332" r="BP76"/>
-      <c s="333" r="BQ76"/>
-      <c s="393" r="BR76"/>
-      <c s="332" r="BS76"/>
-      <c s="334" r="BT76"/>
-      <c s="332" r="BU76"/>
-      <c s="332" r="BV76"/>
-      <c s="324" r="BW76"/>
-      <c s="393" r="BX76"/>
-      <c s="332" r="BY76"/>
-      <c s="333" r="BZ76"/>
-      <c s="393" r="CA76"/>
-      <c s="332" r="CB76"/>
-      <c s="333" r="CC76"/>
-      <c s="393" r="CD76"/>
-      <c s="332" r="CE76"/>
-      <c s="333" r="CF76"/>
-      <c s="393" r="CG76"/>
-      <c s="332" r="CH76"/>
-      <c s="333" r="CI76"/>
-      <c s="393" r="CJ76"/>
-      <c s="332" r="CK76"/>
-      <c s="334" r="CL76"/>
-      <c s="332" r="CM76"/>
-      <c s="332" r="CN76"/>
-      <c s="325" r="CO76"/>
-      <c s="332" r="CP76"/>
-      <c s="332" r="CQ76"/>
-      <c s="326" r="CR76"/>
-      <c s="332" r="CS76"/>
-      <c s="332" r="CT76"/>
-      <c s="326" r="CU76"/>
-      <c s="332" r="CV76"/>
-      <c s="332" r="CW76"/>
-      <c s="326" r="CX76"/>
-      <c s="332" r="CY76"/>
-      <c s="332" r="CZ76"/>
-      <c s="326" r="DA76"/>
-      <c s="332" r="DB76"/>
-      <c s="332" r="DC76"/>
-      <c s="326" r="DD76"/>
-      <c s="332" r="DE76"/>
-      <c s="332" r="DF76"/>
-      <c s="335" r="DG76"/>
+      <c s="995" r="C76"/>
+      <c s="1005" r="D76"/>
+      <c s="998" r="E76"/>
+      <c s="995" r="F76"/>
+      <c s="1005" r="G76"/>
+      <c s="998" r="H76"/>
+      <c s="995" r="I76"/>
+      <c s="1005" r="J76"/>
+      <c s="998" r="K76"/>
+      <c s="995" r="L76"/>
+      <c s="1005" r="M76"/>
+      <c s="998" r="N76"/>
+      <c s="995" r="O76"/>
+      <c s="1005" r="P76"/>
+      <c s="998" r="Q76"/>
+      <c s="995" r="R76"/>
+      <c s="999" r="S76"/>
+      <c s="998" r="T76"/>
+      <c s="995" r="U76"/>
+      <c s="1005" r="V76"/>
+      <c s="998" r="W76"/>
+      <c s="995" r="X76"/>
+      <c s="1005" r="Y76"/>
+      <c s="998" r="Z76"/>
+      <c s="995" r="AA76"/>
+      <c s="1005" r="AB76"/>
+      <c s="998" r="AC76"/>
+      <c s="995" r="AD76"/>
+      <c s="1005" r="AE76"/>
+      <c s="998" r="AF76"/>
+      <c s="995" r="AG76"/>
+      <c s="1005" r="AH76"/>
+      <c s="998" r="AI76"/>
+      <c s="995" r="AJ76"/>
+      <c s="999" r="AK76"/>
+      <c s="998" r="AL76"/>
+      <c s="995" r="AM76"/>
+      <c s="1005" r="AN76"/>
+      <c s="998" r="AO76"/>
+      <c s="995" r="AP76"/>
+      <c s="1005" r="AQ76"/>
+      <c s="998" r="AR76"/>
+      <c s="995" r="AS76"/>
+      <c s="1005" r="AT76"/>
+      <c s="998" r="AU76"/>
+      <c s="995" r="AV76"/>
+      <c s="1005" r="AW76"/>
+      <c s="998" r="AX76"/>
+      <c s="995" r="AY76"/>
+      <c s="1005" r="AZ76"/>
+      <c s="998" r="BA76"/>
+      <c s="995" r="BB76"/>
+      <c s="999" r="BC76"/>
+      <c s="998" r="BD76"/>
+      <c s="995" r="BE76"/>
+      <c s="1005" r="BF76"/>
+      <c s="998" r="BG76"/>
+      <c s="995" r="BH76"/>
+      <c s="1005" r="BI76"/>
+      <c s="998" r="BJ76"/>
+      <c s="995" r="BK76"/>
+      <c s="1005" r="BL76"/>
+      <c s="998" r="BM76"/>
+      <c s="995" r="BN76"/>
+      <c s="1005" r="BO76"/>
+      <c s="998" r="BP76"/>
+      <c s="995" r="BQ76"/>
+      <c s="1005" r="BR76"/>
+      <c s="998" r="BS76"/>
+      <c s="995" r="BT76"/>
+      <c s="999" r="BU76"/>
+      <c s="998" r="BV76"/>
+      <c s="995" r="BW76"/>
+      <c s="1005" r="BX76"/>
+      <c s="998" r="BY76"/>
+      <c s="995" r="BZ76"/>
+      <c s="1005" r="CA76"/>
+      <c s="998" r="CB76"/>
+      <c s="995" r="CC76"/>
+      <c s="1005" r="CD76"/>
+      <c s="998" r="CE76"/>
+      <c s="995" r="CF76"/>
+      <c s="1005" r="CG76"/>
+      <c s="998" r="CH76"/>
+      <c s="995" r="CI76"/>
+      <c s="1005" r="CJ76"/>
+      <c s="998" r="CK76"/>
+      <c s="995" r="CL76"/>
+      <c s="999" r="CM76"/>
+      <c s="998" r="CN76"/>
+      <c s="995" r="CO76"/>
+      <c s="999" r="CP76"/>
+      <c s="998" r="CQ76"/>
+      <c s="995" r="CR76"/>
+      <c s="999" r="CS76"/>
+      <c s="998" r="CT76"/>
+      <c s="995" r="CU76"/>
+      <c s="999" r="CV76"/>
+      <c s="998" r="CW76"/>
+      <c s="995" r="CX76"/>
+      <c s="999" r="CY76"/>
+      <c s="998" r="CZ76"/>
+      <c s="995" r="DA76"/>
+      <c s="999" r="DB76"/>
+      <c s="998" r="DC76"/>
+      <c s="995" r="DD76"/>
+      <c s="999" r="DE76"/>
+      <c s="998" r="DF76"/>
+      <c s="995" r="DG76"/>
     </row>
-    <row r="77" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A77"/>
-      <c s="322" r="B77" t="str">
+    <row r="77" ht="23" customHeight="1">
+      <c s="995" r="A77"/>
+      <c s="1002" r="B77" t="str">
         <v>关税税率</v>
       </c>
-      <c s="331" r="C77"/>
-      <c s="361" r="D77"/>
-      <c s="332" r="E77"/>
-      <c s="333" r="F77"/>
-      <c s="361" r="G77"/>
-      <c s="332" r="H77"/>
-      <c s="333" r="I77"/>
-      <c s="361" r="J77"/>
-      <c s="332" r="K77"/>
-      <c s="333" r="L77"/>
-      <c s="361" r="M77"/>
-      <c s="332" r="N77"/>
-      <c s="333" r="O77"/>
-      <c s="361" r="P77"/>
-      <c s="332" r="Q77"/>
-      <c s="334" r="R77"/>
-      <c s="332" r="S77"/>
-      <c s="332" r="T77"/>
-      <c s="324" r="U77"/>
-      <c s="361" r="V77"/>
-      <c s="332" r="W77"/>
-      <c s="333" r="X77"/>
-      <c s="361" r="Y77"/>
-      <c s="332" r="Z77"/>
-      <c s="333" r="AA77"/>
-      <c s="361" r="AB77"/>
-      <c s="332" r="AC77"/>
-      <c s="333" r="AD77"/>
-      <c s="361" r="AE77"/>
-      <c s="332" r="AF77"/>
-      <c s="333" r="AG77"/>
-      <c s="361" r="AH77"/>
-      <c s="332" r="AI77"/>
-      <c s="334" r="AJ77"/>
-      <c s="332" r="AK77"/>
-      <c s="332" r="AL77"/>
-      <c s="324" r="AM77"/>
-      <c s="361" r="AN77"/>
-      <c s="332" r="AO77"/>
-      <c s="333" r="AP77"/>
-      <c s="361" r="AQ77"/>
-      <c s="332" r="AR77"/>
-      <c s="333" r="AS77"/>
-      <c s="361" r="AT77"/>
-      <c s="332" r="AU77"/>
-      <c s="333" r="AV77"/>
-      <c s="361" r="AW77"/>
-      <c s="332" r="AX77"/>
-      <c s="333" r="AY77"/>
-      <c s="361" r="AZ77"/>
-      <c s="332" r="BA77"/>
-      <c s="334" r="BB77"/>
-      <c s="332" r="BC77"/>
-      <c s="332" r="BD77"/>
-      <c s="324" r="BE77"/>
-      <c s="361" r="BF77"/>
-      <c s="332" r="BG77"/>
-      <c s="333" r="BH77"/>
-      <c s="361" r="BI77"/>
-      <c s="332" r="BJ77"/>
-      <c s="333" r="BK77"/>
-      <c s="361" r="BL77"/>
-      <c s="332" r="BM77"/>
-      <c s="333" r="BN77"/>
-      <c s="361" r="BO77"/>
-      <c s="332" r="BP77"/>
-      <c s="333" r="BQ77"/>
-      <c s="361" r="BR77"/>
-      <c s="332" r="BS77"/>
-      <c s="334" r="BT77"/>
-      <c s="332" r="BU77"/>
-      <c s="332" r="BV77"/>
-      <c s="324" r="BW77"/>
-      <c s="361" r="BX77"/>
-      <c s="332" r="BY77"/>
-      <c s="333" r="BZ77"/>
-      <c s="361" r="CA77"/>
-      <c s="332" r="CB77"/>
-      <c s="333" r="CC77"/>
-      <c s="361" r="CD77"/>
-      <c s="332" r="CE77"/>
-      <c s="333" r="CF77"/>
-      <c s="361" r="CG77"/>
-      <c s="332" r="CH77"/>
-      <c s="333" r="CI77"/>
-      <c s="361" r="CJ77"/>
-      <c s="332" r="CK77"/>
-      <c s="334" r="CL77"/>
-      <c s="332" r="CM77"/>
-      <c s="332" r="CN77"/>
-      <c s="325" r="CO77"/>
-      <c s="332" r="CP77"/>
-      <c s="332" r="CQ77"/>
-      <c s="326" r="CR77"/>
-      <c s="332" r="CS77"/>
-      <c s="332" r="CT77"/>
-      <c s="326" r="CU77"/>
-      <c s="332" r="CV77"/>
-      <c s="332" r="CW77"/>
-      <c s="326" r="CX77"/>
-      <c s="332" r="CY77"/>
-      <c s="332" r="CZ77"/>
-      <c s="326" r="DA77"/>
-      <c s="332" r="DB77"/>
-      <c s="332" r="DC77"/>
-      <c s="326" r="DD77"/>
-      <c s="332" r="DE77"/>
-      <c s="332" r="DF77"/>
-      <c s="335" r="DG77"/>
+      <c s="995" r="C77"/>
+      <c s="1003" r="D77"/>
+      <c s="998" r="E77"/>
+      <c s="995" r="F77"/>
+      <c s="1003" r="G77"/>
+      <c s="998" r="H77"/>
+      <c s="995" r="I77"/>
+      <c s="1003" r="J77"/>
+      <c s="998" r="K77"/>
+      <c s="995" r="L77"/>
+      <c s="1003" r="M77"/>
+      <c s="998" r="N77"/>
+      <c s="995" r="O77"/>
+      <c s="1003" r="P77"/>
+      <c s="998" r="Q77"/>
+      <c s="995" r="R77"/>
+      <c s="1004" r="S77"/>
+      <c s="998" r="T77"/>
+      <c s="995" r="U77"/>
+      <c s="1003" r="V77"/>
+      <c s="998" r="W77"/>
+      <c s="995" r="X77"/>
+      <c s="1003" r="Y77"/>
+      <c s="998" r="Z77"/>
+      <c s="995" r="AA77"/>
+      <c s="1003" r="AB77"/>
+      <c s="998" r="AC77"/>
+      <c s="995" r="AD77"/>
+      <c s="1003" r="AE77"/>
+      <c s="998" r="AF77"/>
+      <c s="995" r="AG77"/>
+      <c s="1003" r="AH77"/>
+      <c s="998" r="AI77"/>
+      <c s="995" r="AJ77"/>
+      <c s="1004" r="AK77"/>
+      <c s="998" r="AL77"/>
+      <c s="995" r="AM77"/>
+      <c s="1003" r="AN77"/>
+      <c s="998" r="AO77"/>
+      <c s="995" r="AP77"/>
+      <c s="1003" r="AQ77"/>
+      <c s="998" r="AR77"/>
+      <c s="995" r="AS77"/>
+      <c s="1003" r="AT77"/>
+      <c s="998" r="AU77"/>
+      <c s="995" r="AV77"/>
+      <c s="1003" r="AW77"/>
+      <c s="998" r="AX77"/>
+      <c s="995" r="AY77"/>
+      <c s="1003" r="AZ77"/>
+      <c s="998" r="BA77"/>
+      <c s="995" r="BB77"/>
+      <c s="1004" r="BC77"/>
+      <c s="998" r="BD77"/>
+      <c s="995" r="BE77"/>
+      <c s="1003" r="BF77"/>
+      <c s="998" r="BG77"/>
+      <c s="995" r="BH77"/>
+      <c s="1003" r="BI77"/>
+      <c s="998" r="BJ77"/>
+      <c s="995" r="BK77"/>
+      <c s="1003" r="BL77"/>
+      <c s="998" r="BM77"/>
+      <c s="995" r="BN77"/>
+      <c s="1003" r="BO77"/>
+      <c s="998" r="BP77"/>
+      <c s="995" r="BQ77"/>
+      <c s="1003" r="BR77"/>
+      <c s="998" r="BS77"/>
+      <c s="995" r="BT77"/>
+      <c s="1004" r="BU77"/>
+      <c s="998" r="BV77"/>
+      <c s="995" r="BW77"/>
+      <c s="1003" r="BX77"/>
+      <c s="998" r="BY77"/>
+      <c s="995" r="BZ77"/>
+      <c s="1003" r="CA77"/>
+      <c s="998" r="CB77"/>
+      <c s="995" r="CC77"/>
+      <c s="1003" r="CD77"/>
+      <c s="998" r="CE77"/>
+      <c s="995" r="CF77"/>
+      <c s="1003" r="CG77"/>
+      <c s="998" r="CH77"/>
+      <c s="995" r="CI77"/>
+      <c s="1003" r="CJ77"/>
+      <c s="998" r="CK77"/>
+      <c s="995" r="CL77"/>
+      <c s="1004" r="CM77"/>
+      <c s="998" r="CN77"/>
+      <c s="995" r="CO77"/>
+      <c s="1004" r="CP77"/>
+      <c s="998" r="CQ77"/>
+      <c s="995" r="CR77"/>
+      <c s="1004" r="CS77"/>
+      <c s="998" r="CT77"/>
+      <c s="995" r="CU77"/>
+      <c s="1004" r="CV77"/>
+      <c s="998" r="CW77"/>
+      <c s="995" r="CX77"/>
+      <c s="1004" r="CY77"/>
+      <c s="998" r="CZ77"/>
+      <c s="995" r="DA77"/>
+      <c s="1004" r="DB77"/>
+      <c s="998" r="DC77"/>
+      <c s="995" r="DD77"/>
+      <c s="1004" r="DE77"/>
+      <c s="998" r="DF77"/>
+      <c s="995" r="DG77"/>
     </row>
-    <row r="78" spans="1:111" ht="23" customHeight="1">
-      <c s="321" r="A78"/>
-      <c s="322" r="B78" t="str">
+    <row r="78" ht="23" customHeight="1">
+      <c s="995" r="A78"/>
+      <c s="1002" r="B78" t="str">
         <v>质保计提比例（按 MSRP）</v>
       </c>
-      <c s="331" r="C78"/>
-      <c s="361" r="D78"/>
-      <c s="332" r="E78"/>
-      <c s="333" r="F78"/>
-      <c s="361" r="G78"/>
-      <c s="332" r="H78"/>
-      <c s="333" r="I78"/>
-      <c s="361" r="J78"/>
-      <c s="332" r="K78"/>
-      <c s="333" r="L78"/>
-      <c s="361" r="M78"/>
-      <c s="332" r="N78"/>
-      <c s="333" r="O78"/>
-      <c s="361" r="P78"/>
-      <c s="332" r="Q78"/>
-      <c s="334" r="R78"/>
-      <c s="332" r="S78"/>
-      <c s="332" r="T78"/>
-      <c s="324" r="U78"/>
-      <c s="361" r="V78"/>
-      <c s="332" r="W78"/>
-      <c s="333" r="X78"/>
-      <c s="361" r="Y78"/>
-      <c s="332" r="Z78"/>
-      <c s="333" r="AA78"/>
-      <c s="361" r="AB78"/>
-      <c s="332" r="AC78"/>
-      <c s="333" r="AD78"/>
-      <c s="361" r="AE78"/>
-      <c s="332" r="AF78"/>
-      <c s="333" r="AG78"/>
-      <c s="361" r="AH78"/>
-      <c s="332" r="AI78"/>
-      <c s="334" r="AJ78"/>
-      <c s="332" r="AK78"/>
-      <c s="332" r="AL78"/>
-      <c s="324" r="AM78"/>
-      <c s="361" r="AN78"/>
-      <c s="332" r="AO78"/>
-      <c s="333" r="AP78"/>
-      <c s="361" r="AQ78"/>
-      <c s="332" r="AR78"/>
-      <c s="333" r="AS78"/>
-      <c s="361" r="AT78"/>
-      <c s="332" r="AU78"/>
-      <c s="333" r="AV78"/>
-      <c s="361" r="AW78"/>
-      <c s="332" r="AX78"/>
-      <c s="333" r="AY78"/>
-      <c s="361" r="AZ78"/>
-      <c s="332" r="BA78"/>
-      <c s="334" r="BB78"/>
-      <c s="332" r="BC78"/>
-      <c s="332" r="BD78"/>
-      <c s="324" r="BE78"/>
-      <c s="361" r="BF78"/>
-      <c s="332" r="BG78"/>
-      <c s="333" r="BH78"/>
-      <c s="361" r="BI78"/>
-      <c s="332" r="BJ78"/>
-      <c s="333" r="BK78"/>
-      <c s="361" r="BL78"/>
-      <c s="332" r="BM78"/>
-      <c s="333" r="BN78"/>
-      <c s="361" r="BO78"/>
-      <c s="332" r="BP78"/>
-      <c s="333" r="BQ78"/>
-      <c s="361" r="BR78"/>
-      <c s="332" r="BS78"/>
-      <c s="334" r="BT78"/>
-      <c s="332" r="BU78"/>
-      <c s="332" r="BV78"/>
-      <c s="324" r="BW78"/>
-      <c s="361" r="BX78"/>
-      <c s="332" r="BY78"/>
-      <c s="333" r="BZ78"/>
-      <c s="361" r="CA78"/>
-      <c s="332" r="CB78"/>
-      <c s="333" r="CC78"/>
-      <c s="361" r="CD78"/>
-      <c s="332" r="CE78"/>
-      <c s="333" r="CF78"/>
-      <c s="361" r="CG78"/>
-      <c s="332" r="CH78"/>
-      <c s="333" r="CI78"/>
-      <c s="361" r="CJ78"/>
-      <c s="332" r="CK78"/>
-      <c s="334" r="CL78"/>
-      <c s="332" r="CM78"/>
-      <c s="332" r="CN78"/>
-      <c s="325" r="CO78"/>
-      <c s="332" r="CP78"/>
-      <c s="332" r="CQ78"/>
-      <c s="326" r="CR78"/>
-      <c s="332" r="CS78"/>
-      <c s="332" r="CT78"/>
-      <c s="326" r="CU78"/>
-      <c s="332" r="CV78"/>
-      <c s="332" r="CW78"/>
-      <c s="326" r="CX78"/>
-      <c s="332" r="CY78"/>
-      <c s="332" r="CZ78"/>
-      <c s="326" r="DA78"/>
-      <c s="332" r="DB78"/>
-      <c s="332" r="DC78"/>
-      <c s="326" r="DD78"/>
-      <c s="332" r="DE78"/>
-      <c s="332" r="DF78"/>
-      <c s="335" r="DG78"/>
+      <c s="995" r="C78"/>
+      <c s="1003" r="D78"/>
+      <c s="998" r="E78"/>
+      <c s="995" r="F78"/>
+      <c s="1003" r="G78"/>
+      <c s="998" r="H78"/>
+      <c s="995" r="I78"/>
+      <c s="1003" r="J78"/>
+      <c s="998" r="K78"/>
+      <c s="995" r="L78"/>
+      <c s="1003" r="M78"/>
+      <c s="998" r="N78"/>
+      <c s="995" r="O78"/>
+      <c s="1003" r="P78"/>
+      <c s="998" r="Q78"/>
+      <c s="995" r="R78"/>
+      <c s="1004" r="S78"/>
+      <c s="998" r="T78"/>
+      <c s="995" r="U78"/>
+      <c s="1003" r="V78"/>
+      <c s="998" r="W78"/>
+      <c s="995" r="X78"/>
+      <c s="1003" r="Y78"/>
+      <c s="998" r="Z78"/>
+      <c s="995" r="AA78"/>
+      <c s="1003" r="AB78"/>
+      <c s="998" r="AC78"/>
+      <c s="995" r="AD78"/>
+      <c s="1003" r="AE78"/>
+      <c s="998" r="AF78"/>
+      <c s="995" r="AG78"/>
+      <c s="1003" r="AH78"/>
+      <c s="998" r="AI78"/>
+      <c s="995" r="AJ78"/>
+      <c s="1004" r="AK78"/>
+      <c s="998" r="AL78"/>
+      <c s="995" r="AM78"/>
+      <c s="1003" r="AN78"/>
+      <c s="998" r="AO78"/>
+      <c s="995" r="AP78"/>
+      <c s="1003" r="AQ78"/>
+      <c s="998" r="AR78"/>
+      <c s="995" r="AS78"/>
+      <c s="1003" r="AT78"/>
+      <c s="998" r="AU78"/>
+      <c s="995" r="AV78"/>
+      <c s="1003" r="AW78"/>
+      <c s="998" r="AX78"/>
+      <c s="995" r="AY78"/>
+      <c s="1003" r="AZ78"/>
+      <c s="998" r="BA78"/>
+      <c s="995" r="BB78"/>
+      <c s="1004" r="BC78"/>
+      <c s="998" r="BD78"/>
+      <c s="995" r="BE78"/>
+      <c s="1003" r="BF78"/>
+      <c s="998" r="BG78"/>
+      <c s="995" r="BH78"/>
+      <c s="1003" r="BI78"/>
+      <c s="998" r="BJ78"/>
+      <c s="995" r="BK78"/>
+      <c s="1003" r="BL78"/>
+      <c s="998" r="BM78"/>
+      <c s="995" r="BN78"/>
+      <c s="1003" r="BO78"/>
+      <c s="998" r="BP78"/>
+      <c s="995" r="BQ78"/>
+      <c s="1003" r="BR78"/>
+      <c s="998" r="BS78"/>
+      <c s="995" r="BT78"/>
+      <c s="1004" r="BU78"/>
+      <c s="998" r="BV78"/>
+      <c s="995" r="BW78"/>
+      <c s="1003" r="BX78"/>
+      <c s="998" r="BY78"/>
+      <c s="995" r="BZ78"/>
+      <c s="1003" r="CA78"/>
+      <c s="998" r="CB78"/>
+      <c s="995" r="CC78"/>
+      <c s="1003" r="CD78"/>
+      <c s="998" r="CE78"/>
+      <c s="995" r="CF78"/>
+      <c s="1003" r="CG78"/>
+      <c s="998" r="CH78"/>
+      <c s="995" r="CI78"/>
+      <c s="1003" r="CJ78"/>
+      <c s="998" r="CK78"/>
+      <c s="995" r="CL78"/>
+      <c s="1004" r="CM78"/>
+      <c s="998" r="CN78"/>
+      <c s="995" r="CO78"/>
+      <c s="1004" r="CP78"/>
+      <c s="998" r="CQ78"/>
+      <c s="995" r="CR78"/>
+      <c s="1004" r="CS78"/>
+      <c s="998" r="CT78"/>
+      <c s="995" r="CU78"/>
+      <c s="1004" r="CV78"/>
+      <c s="998" r="CW78"/>
+      <c s="995" r="CX78"/>
+      <c s="1004" r="CY78"/>
+      <c s="998" r="CZ78"/>
+      <c s="995" r="DA78"/>
+      <c s="1004" r="DB78"/>
+      <c s="998" r="DC78"/>
+      <c s="995" r="DD78"/>
+      <c s="1004" r="DE78"/>
+      <c s="998" r="DF78"/>
+      <c s="995" r="DG78"/>
     </row>
-    <row r="79" spans="1:111" ht="22" customHeight="1">
-      <c s="321" r="A79"/>
-      <c s="322" r="B79"/>
-      <c s="331" r="C79"/>
-      <c s="332" r="D79"/>
-      <c s="332" r="E79"/>
-      <c s="333" r="F79"/>
-      <c s="332" r="G79"/>
-      <c s="332" r="H79"/>
-      <c s="333" r="I79"/>
-      <c s="332" r="J79"/>
-      <c s="332" r="K79"/>
-      <c s="333" r="L79"/>
-      <c s="332" r="M79"/>
-      <c s="332" r="N79"/>
-      <c s="333" r="O79"/>
-      <c s="332" r="P79"/>
-      <c s="332" r="Q79"/>
-      <c s="334" r="R79"/>
-      <c s="332" r="S79"/>
-      <c s="332" r="T79"/>
-      <c s="324" r="U79"/>
-      <c s="332" r="V79"/>
-      <c s="332" r="W79"/>
-      <c s="333" r="X79"/>
-      <c s="332" r="Y79"/>
-      <c s="332" r="Z79"/>
-      <c s="333" r="AA79"/>
-      <c s="332" r="AB79"/>
-      <c s="332" r="AC79"/>
-      <c s="333" r="AD79"/>
-      <c s="332" r="AE79"/>
-      <c s="332" r="AF79"/>
-      <c s="333" r="AG79"/>
-      <c s="332" r="AH79"/>
-      <c s="332" r="AI79"/>
-      <c s="334" r="AJ79"/>
-      <c s="332" r="AK79"/>
-      <c s="332" r="AL79"/>
-      <c s="324" r="AM79"/>
-      <c s="332" r="AN79"/>
-      <c s="332" r="AO79"/>
-      <c s="333" r="AP79"/>
-      <c s="332" r="AQ79"/>
-      <c s="332" r="AR79"/>
-      <c s="333" r="AS79"/>
-      <c s="332" r="AT79"/>
-      <c s="332" r="AU79"/>
-      <c s="333" r="AV79"/>
-      <c s="332" r="AW79"/>
-      <c s="332" r="AX79"/>
-      <c s="333" r="AY79"/>
-      <c s="332" r="AZ79"/>
-      <c s="332" r="BA79"/>
-      <c s="334" r="BB79"/>
-      <c s="332" r="BC79"/>
-      <c s="332" r="BD79"/>
-      <c s="324" r="BE79"/>
-      <c s="332" r="BF79"/>
-      <c s="332" r="BG79"/>
-      <c s="333" r="BH79"/>
-      <c s="332" r="BI79"/>
-      <c s="332" r="BJ79"/>
-      <c s="333" r="BK79"/>
-      <c s="332" r="BL79"/>
-      <c s="332" r="BM79"/>
-      <c s="333" r="BN79"/>
-      <c s="332" r="BO79"/>
-      <c s="332" r="BP79"/>
-      <c s="333" r="BQ79"/>
-      <c s="332" r="BR79"/>
-      <c s="332" r="BS79"/>
-      <c s="334" r="BT79"/>
-      <c s="332" r="BU79"/>
-      <c s="332" r="BV79"/>
-      <c s="324" r="BW79"/>
-      <c s="332" r="BX79"/>
-      <c s="332" r="BY79"/>
-      <c s="333" r="BZ79"/>
-      <c s="332" r="CA79"/>
-      <c s="332" r="CB79"/>
-      <c s="333" r="CC79"/>
-      <c s="332" r="CD79"/>
-      <c s="332" r="CE79"/>
-      <c s="333" r="CF79"/>
-      <c s="332" r="CG79"/>
-      <c s="332" r="CH79"/>
-      <c s="333" r="CI79"/>
-      <c s="332" r="CJ79"/>
-      <c s="332" r="CK79"/>
-      <c s="334" r="CL79"/>
-      <c s="332" r="CM79"/>
-      <c s="332" r="CN79"/>
-      <c s="325" r="CO79"/>
-      <c s="332" r="CP79"/>
-      <c s="332" r="CQ79"/>
-      <c s="326" r="CR79"/>
-      <c s="332" r="CS79"/>
-      <c s="332" r="CT79"/>
-      <c s="326" r="CU79"/>
-      <c s="332" r="CV79"/>
-      <c s="332" r="CW79"/>
-      <c s="326" r="CX79"/>
-      <c s="332" r="CY79"/>
-      <c s="332" r="CZ79"/>
-      <c s="326" r="DA79"/>
-      <c s="332" r="DB79"/>
-      <c s="332" r="DC79"/>
-      <c s="326" r="DD79"/>
-      <c s="332" r="DE79"/>
-      <c s="332" r="DF79"/>
-      <c s="335" r="DG79"/>
+    <row r="79" ht="22" customHeight="1">
+      <c s="995" r="A79"/>
+      <c s="996" r="B79"/>
+      <c s="995" r="C79"/>
+      <c s="997" r="D79"/>
+      <c s="998" r="E79"/>
+      <c s="995" r="F79"/>
+      <c s="997" r="G79"/>
+      <c s="998" r="H79"/>
+      <c s="995" r="I79"/>
+      <c s="997" r="J79"/>
+      <c s="998" r="K79"/>
+      <c s="995" r="L79"/>
+      <c s="997" r="M79"/>
+      <c s="998" r="N79"/>
+      <c s="995" r="O79"/>
+      <c s="997" r="P79"/>
+      <c s="998" r="Q79"/>
+      <c s="995" r="R79"/>
+      <c s="999" r="S79"/>
+      <c s="998" r="T79"/>
+      <c s="995" r="U79"/>
+      <c s="997" r="V79"/>
+      <c s="998" r="W79"/>
+      <c s="995" r="X79"/>
+      <c s="997" r="Y79"/>
+      <c s="998" r="Z79"/>
+      <c s="995" r="AA79"/>
+      <c s="997" r="AB79"/>
+      <c s="998" r="AC79"/>
+      <c s="995" r="AD79"/>
+      <c s="997" r="AE79"/>
+      <c s="998" r="AF79"/>
+      <c s="995" r="AG79"/>
+      <c s="997" r="AH79"/>
+      <c s="998" r="AI79"/>
+      <c s="995" r="AJ79"/>
+      <c s="999" r="AK79"/>
+      <c s="998" r="AL79"/>
+      <c s="995" r="AM79"/>
+      <c s="997" r="AN79"/>
+      <c s="998" r="AO79"/>
+      <c s="995" r="AP79"/>
+      <c s="997" r="AQ79"/>
+      <c s="998" r="AR79"/>
+      <c s="995" r="AS79"/>
+      <c s="997" r="AT79"/>
+      <c s="998" r="AU79"/>
+      <c s="995" r="AV79"/>
+      <c s="997" r="AW79"/>
+      <c s="998" r="AX79"/>
+      <c s="995" r="AY79"/>
+      <c s="997" r="AZ79"/>
+      <c s="998" r="BA79"/>
+      <c s="995" r="BB79"/>
+      <c s="999" r="BC79"/>
+      <c s="998" r="BD79"/>
+      <c s="995" r="BE79"/>
+      <c s="997" r="BF79"/>
+      <c s="998" r="BG79"/>
+      <c s="995" r="BH79"/>
+      <c s="997" r="BI79"/>
+      <c s="998" r="BJ79"/>
+      <c s="995" r="BK79"/>
+      <c s="997" r="BL79"/>
+      <c s="998" r="BM79"/>
+      <c s="995" r="BN79"/>
+      <c s="997" r="BO79"/>
+      <c s="998" r="BP79"/>
+      <c s="995" r="BQ79"/>
+      <c s="997" r="BR79"/>
+      <c s="998" r="BS79"/>
+      <c s="995" r="BT79"/>
+      <c s="999" r="BU79"/>
+      <c s="998" r="BV79"/>
+      <c s="995" r="BW79"/>
+      <c s="997" r="BX79"/>
+      <c s="998" r="BY79"/>
+      <c s="995" r="BZ79"/>
+      <c s="997" r="CA79"/>
+      <c s="998" r="CB79"/>
+      <c s="995" r="CC79"/>
+      <c s="997" r="CD79"/>
+      <c s="998" r="CE79"/>
+      <c s="995" r="CF79"/>
+      <c s="997" r="CG79"/>
+      <c s="998" r="CH79"/>
+      <c s="995" r="CI79"/>
+      <c s="997" r="CJ79"/>
+      <c s="998" r="CK79"/>
+      <c s="995" r="CL79"/>
+      <c s="999" r="CM79"/>
+      <c s="998" r="CN79"/>
+      <c s="995" r="CO79"/>
+      <c s="999" r="CP79"/>
+      <c s="998" r="CQ79"/>
+      <c s="995" r="CR79"/>
+      <c s="999" r="CS79"/>
+      <c s="998" r="CT79"/>
+      <c s="995" r="CU79"/>
+      <c s="999" r="CV79"/>
+      <c s="998" r="CW79"/>
+      <c s="995" r="CX79"/>
+      <c s="999" r="CY79"/>
+      <c s="998" r="CZ79"/>
+      <c s="995" r="DA79"/>
+      <c s="999" r="DB79"/>
+      <c s="998" r="DC79"/>
+      <c s="995" r="DD79"/>
+      <c s="999" r="DE79"/>
+      <c s="998" r="DF79"/>
+      <c s="995" r="DG79"/>
     </row>
-    <row r="80" spans="1:111" ht="22" customHeight="1">
-      <c s="321" r="A80"/>
-      <c s="343" r="B80"/>
-      <c s="331" r="C80"/>
-      <c s="332" r="D80"/>
-      <c s="332" r="E80"/>
-      <c s="333" r="F80"/>
-      <c s="332" r="G80"/>
-      <c s="332" r="H80"/>
-      <c s="333" r="I80"/>
-      <c s="332" r="J80"/>
-      <c s="332" r="K80"/>
-      <c s="333" r="L80"/>
-      <c s="332" r="M80"/>
-      <c s="332" r="N80"/>
-      <c s="333" r="O80"/>
-      <c s="332" r="P80"/>
-      <c s="332" r="Q80"/>
-      <c s="334" r="R80"/>
-      <c s="332" r="S80"/>
-      <c s="332" r="T80"/>
-      <c s="324" r="U80"/>
-      <c s="332" r="V80"/>
-      <c s="332" r="W80"/>
-      <c s="333" r="X80"/>
-      <c s="332" r="Y80"/>
-      <c s="332" r="Z80"/>
-      <c s="333" r="AA80"/>
-      <c s="332" r="AB80"/>
-      <c s="332" r="AC80"/>
-      <c s="333" r="AD80"/>
-      <c s="332" r="AE80"/>
-      <c s="332" r="AF80"/>
-      <c s="333" r="AG80"/>
-      <c s="332" r="AH80"/>
-      <c s="332" r="AI80"/>
-      <c s="334" r="AJ80"/>
-      <c s="332" r="AK80"/>
-      <c s="332" r="AL80"/>
-      <c s="324" r="AM80"/>
-      <c s="332" r="AN80"/>
-      <c s="332" r="AO80"/>
-      <c s="333" r="AP80"/>
-      <c s="332" r="AQ80"/>
-      <c s="332" r="AR80"/>
-      <c s="333" r="AS80"/>
-      <c s="332" r="AT80"/>
-      <c s="332" r="AU80"/>
-      <c s="333" r="AV80"/>
-      <c s="332" r="AW80"/>
-      <c s="332" r="AX80"/>
-      <c s="333" r="AY80"/>
-      <c s="332" r="AZ80"/>
-      <c s="332" r="BA80"/>
-      <c s="334" r="BB80"/>
-      <c s="332" r="BC80"/>
-      <c s="332" r="BD80"/>
-      <c s="324" r="BE80"/>
-      <c s="332" r="BF80"/>
-      <c s="332" r="BG80"/>
-      <c s="333" r="BH80"/>
-      <c s="332" r="BI80"/>
-      <c s="332" r="BJ80"/>
-      <c s="333" r="BK80"/>
-      <c s="332" r="BL80"/>
-      <c s="332" r="BM80"/>
-      <c s="333" r="BN80"/>
-      <c s="332" r="BO80"/>
-      <c s="332" r="BP80"/>
-      <c s="333" r="BQ80"/>
-      <c s="332" r="BR80"/>
-      <c s="332" r="BS80"/>
-      <c s="334" r="BT80"/>
-      <c s="332" r="BU80"/>
-      <c s="332" r="BV80"/>
-      <c s="324" r="BW80"/>
-      <c s="332" r="BX80"/>
-      <c s="332" r="BY80"/>
-      <c s="333" r="BZ80"/>
-      <c s="332" r="CA80"/>
-      <c s="332" r="CB80"/>
-      <c s="333" r="CC80"/>
-      <c s="332" r="CD80"/>
-      <c s="332" r="CE80"/>
-      <c s="333" r="CF80"/>
-      <c s="332" r="CG80"/>
-      <c s="332" r="CH80"/>
-      <c s="333" r="CI80"/>
-      <c s="332" r="CJ80"/>
-      <c s="332" r="CK80"/>
-      <c s="334" r="CL80"/>
-      <c s="332" r="CM80"/>
-      <c s="332" r="CN80"/>
-      <c s="325" r="CO80"/>
-      <c s="332" r="CP80"/>
-      <c s="332" r="CQ80"/>
-      <c s="326" r="CR80"/>
-      <c s="332" r="CS80"/>
-      <c s="332" r="CT80"/>
-      <c s="326" r="CU80"/>
-      <c s="332" r="CV80"/>
-      <c s="332" r="CW80"/>
-      <c s="326" r="CX80"/>
-      <c s="332" r="CY80"/>
-      <c s="332" r="CZ80"/>
-      <c s="326" r="DA80"/>
-      <c s="332" r="DB80"/>
-      <c s="332" r="DC80"/>
-      <c s="326" r="DD80"/>
-      <c s="332" r="DE80"/>
-      <c s="332" r="DF80"/>
-      <c s="335" r="DG80"/>
+    <row r="80" ht="22" customHeight="1">
+      <c s="995" r="A80"/>
+      <c s="996" r="B80"/>
+      <c s="995" r="C80"/>
+      <c s="997" r="D80"/>
+      <c s="998" r="E80"/>
+      <c s="995" r="F80"/>
+      <c s="997" r="G80"/>
+      <c s="998" r="H80"/>
+      <c s="995" r="I80"/>
+      <c s="997" r="J80"/>
+      <c s="998" r="K80"/>
+      <c s="995" r="L80"/>
+      <c s="997" r="M80"/>
+      <c s="998" r="N80"/>
+      <c s="995" r="O80"/>
+      <c s="997" r="P80"/>
+      <c s="998" r="Q80"/>
+      <c s="995" r="R80"/>
+      <c s="999" r="S80"/>
+      <c s="998" r="T80"/>
+      <c s="995" r="U80"/>
+      <c s="997" r="V80"/>
+      <c s="998" r="W80"/>
+      <c s="995" r="X80"/>
+      <c s="997" r="Y80"/>
+      <c s="998" r="Z80"/>
+      <c s="995" r="AA80"/>
+      <c s="997" r="AB80"/>
+      <c s="998" r="AC80"/>
+      <c s="995" r="AD80"/>
+      <c s="997" r="AE80"/>
+      <c s="998" r="AF80"/>
+      <c s="995" r="AG80"/>
+      <c s="997" r="AH80"/>
+      <c s="998" r="AI80"/>
+      <c s="995" r="AJ80"/>
+      <c s="999" r="AK80"/>
+      <c s="998" r="AL80"/>
+      <c s="995" r="AM80"/>
+      <c s="997" r="AN80"/>
+      <c s="998" r="AO80"/>
+      <c s="995" r="AP80"/>
+      <c s="997" r="AQ80"/>
+      <c s="998" r="AR80"/>
+      <c s="995" r="AS80"/>
+      <c s="997" r="AT80"/>
+      <c s="998" r="AU80"/>
+      <c s="995" r="AV80"/>
+      <c s="997" r="AW80"/>
+      <c s="998" r="AX80"/>
+      <c s="995" r="AY80"/>
+      <c s="997" r="AZ80"/>
+      <c s="998" r="BA80"/>
+      <c s="995" r="BB80"/>
+      <c s="999" r="BC80"/>
+      <c s="998" r="BD80"/>
+      <c s="995" r="BE80"/>
+      <c s="997" r="BF80"/>
+      <c s="998" r="BG80"/>
+      <c s="995" r="BH80"/>
+      <c s="997" r="BI80"/>
+      <c s="998" r="BJ80"/>
+      <c s="995" r="BK80"/>
+      <c s="997" r="BL80"/>
+      <c s="998" r="BM80"/>
+      <c s="995" r="BN80"/>
+      <c s="997" r="BO80"/>
+      <c s="998" r="BP80"/>
+      <c s="995" r="BQ80"/>
+      <c s="997" r="BR80"/>
+      <c s="998" r="BS80"/>
+      <c s="995" r="BT80"/>
+      <c s="999" r="BU80"/>
+      <c s="998" r="BV80"/>
+      <c s="995" r="BW80"/>
+      <c s="997" r="BX80"/>
+      <c s="998" r="BY80"/>
+      <c s="995" r="BZ80"/>
+      <c s="997" r="CA80"/>
+      <c s="998" r="CB80"/>
+      <c s="995" r="CC80"/>
+      <c s="997" r="CD80"/>
+      <c s="998" r="CE80"/>
+      <c s="995" r="CF80"/>
+      <c s="997" r="CG80"/>
+      <c s="998" r="CH80"/>
+      <c s="995" r="CI80"/>
+      <c s="997" r="CJ80"/>
+      <c s="998" r="CK80"/>
+      <c s="995" r="CL80"/>
+      <c s="999" r="CM80"/>
+      <c s="998" r="CN80"/>
+      <c s="995" r="CO80"/>
+      <c s="999" r="CP80"/>
+      <c s="998" r="CQ80"/>
+      <c s="995" r="CR80"/>
+      <c s="999" r="CS80"/>
+      <c s="998" r="CT80"/>
+      <c s="995" r="CU80"/>
+      <c s="999" r="CV80"/>
+      <c s="998" r="CW80"/>
+      <c s="995" r="CX80"/>
+      <c s="999" r="CY80"/>
+      <c s="998" r="CZ80"/>
+      <c s="995" r="DA80"/>
+      <c s="999" r="DB80"/>
+      <c s="998" r="DC80"/>
+      <c s="995" r="DD80"/>
+      <c s="999" r="DE80"/>
+      <c s="998" r="DF80"/>
+      <c s="995" r="DG80"/>
     </row>
-    <row r="81" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A81"/>
-      <c s="322" r="B81" t="str">
+    <row r="81" ht="24" customHeight="1">
+      <c s="995" r="A81"/>
+      <c s="1006" r="B81" t="str">
         <v>填写方式</v>
       </c>
-      <c s="331" r="C81"/>
-      <c s="332" r="D81" t="str">
+      <c s="995" r="C81"/>
+      <c s="1001" r="D81" t="str">
         <v>填写各年度车型“单车（元）”列。%收入、Average及全生命周期沿用原表展示口径，上传时忽略。</v>
       </c>
-      <c s="332" r="E81"/>
-      <c s="333" r="F81"/>
-      <c s="332" r="G81"/>
-      <c s="332" r="H81"/>
-      <c s="333" r="I81"/>
-      <c s="332" r="J81"/>
-      <c s="332" r="K81"/>
-      <c s="333" r="L81"/>
-      <c s="332" r="M81"/>
-      <c s="332" r="N81"/>
-      <c s="333" r="O81"/>
-      <c s="332" r="P81"/>
-      <c s="332" r="Q81"/>
-      <c s="334" r="R81"/>
-      <c s="332" r="S81"/>
-      <c s="332" r="T81"/>
-      <c s="324" r="U81"/>
-      <c s="332" r="V81"/>
-      <c s="332" r="W81"/>
-      <c s="333" r="X81"/>
-      <c s="332" r="Y81"/>
-      <c s="332" r="Z81"/>
-      <c s="333" r="AA81"/>
-      <c s="332" r="AB81"/>
-      <c s="332" r="AC81"/>
-      <c s="333" r="AD81"/>
-      <c s="332" r="AE81"/>
-      <c s="332" r="AF81"/>
-      <c s="333" r="AG81"/>
-      <c s="332" r="AH81"/>
-      <c s="332" r="AI81"/>
-      <c s="334" r="AJ81"/>
-      <c s="332" r="AK81"/>
-      <c s="332" r="AL81"/>
-      <c s="324" r="AM81"/>
-      <c s="332" r="AN81"/>
-      <c s="332" r="AO81"/>
-      <c s="333" r="AP81"/>
-      <c s="332" r="AQ81"/>
-      <c s="332" r="AR81"/>
-      <c s="333" r="AS81"/>
-      <c s="332" r="AT81"/>
-      <c s="332" r="AU81"/>
-      <c s="333" r="AV81"/>
-      <c s="332" r="AW81"/>
-      <c s="332" r="AX81"/>
-      <c s="333" r="AY81"/>
-      <c s="332" r="AZ81"/>
-      <c s="332" r="BA81"/>
-      <c s="334" r="BB81"/>
-      <c s="332" r="BC81"/>
-      <c s="332" r="BD81"/>
-      <c s="324" r="BE81"/>
-      <c s="332" r="BF81"/>
-      <c s="332" r="BG81"/>
-      <c s="333" r="BH81"/>
-      <c s="332" r="BI81"/>
-      <c s="332" r="BJ81"/>
-      <c s="333" r="BK81"/>
-      <c s="332" r="BL81"/>
-      <c s="332" r="BM81"/>
-      <c s="333" r="BN81"/>
-      <c s="332" r="BO81"/>
-      <c s="332" r="BP81"/>
-      <c s="333" r="BQ81"/>
-      <c s="332" r="BR81"/>
-      <c s="332" r="BS81"/>
-      <c s="334" r="BT81"/>
-      <c s="332" r="BU81"/>
-      <c s="332" r="BV81"/>
-      <c s="324" r="BW81"/>
-      <c s="332" r="BX81"/>
-      <c s="332" r="BY81"/>
-      <c s="333" r="BZ81"/>
-      <c s="332" r="CA81"/>
-      <c s="332" r="CB81"/>
-      <c s="333" r="CC81"/>
-      <c s="332" r="CD81"/>
-      <c s="332" r="CE81"/>
-      <c s="333" r="CF81"/>
-      <c s="332" r="CG81"/>
-      <c s="332" r="CH81"/>
-      <c s="333" r="CI81"/>
-      <c s="332" r="CJ81"/>
-      <c s="332" r="CK81"/>
-      <c s="334" r="CL81"/>
-      <c s="332" r="CM81"/>
-      <c s="332" r="CN81"/>
-      <c s="325" r="CO81"/>
-      <c s="332" r="CP81"/>
-      <c s="332" r="CQ81"/>
-      <c s="326" r="CR81"/>
-      <c s="332" r="CS81"/>
-      <c s="332" r="CT81"/>
-      <c s="326" r="CU81"/>
-      <c s="332" r="CV81"/>
-      <c s="332" r="CW81"/>
-      <c s="326" r="CX81"/>
-      <c s="332" r="CY81"/>
-      <c s="332" r="CZ81"/>
-      <c s="326" r="DA81"/>
-      <c s="332" r="DB81"/>
-      <c s="332" r="DC81"/>
-      <c s="326" r="DD81"/>
-      <c s="332" r="DE81"/>
-      <c s="332" r="DF81"/>
-      <c s="335" r="DG81"/>
+      <c s="1001" r="E81"/>
+      <c s="1001" r="F81"/>
+      <c s="1001" r="G81"/>
+      <c s="1001" r="H81"/>
+      <c s="1001" r="I81"/>
+      <c s="1001" r="J81"/>
+      <c s="1001" r="K81"/>
+      <c s="1001" r="L81"/>
+      <c s="1001" r="M81"/>
+      <c s="1001" r="N81"/>
+      <c s="1001" r="O81"/>
+      <c s="1001" r="P81"/>
+      <c s="1001" r="Q81"/>
+      <c s="1001" r="R81"/>
+      <c s="1001" r="S81"/>
+      <c s="1001" r="T81"/>
+      <c s="995" r="U81"/>
+      <c s="995" r="V81"/>
+      <c s="995" r="W81"/>
+      <c s="995" r="X81"/>
+      <c s="995" r="Y81"/>
+      <c s="995" r="Z81"/>
+      <c s="995" r="AA81"/>
+      <c s="995" r="AB81"/>
+      <c s="995" r="AC81"/>
+      <c s="995" r="AD81"/>
+      <c s="995" r="AE81"/>
+      <c s="995" r="AF81"/>
+      <c s="995" r="AG81"/>
+      <c s="995" r="AH81"/>
+      <c s="995" r="AI81"/>
+      <c s="995" r="AJ81"/>
+      <c s="995" r="AK81"/>
+      <c s="995" r="AL81"/>
+      <c s="995" r="AM81"/>
+      <c s="995" r="AN81"/>
+      <c s="995" r="AO81"/>
+      <c s="995" r="AP81"/>
+      <c s="995" r="AQ81"/>
+      <c s="995" r="AR81"/>
+      <c s="995" r="AS81"/>
+      <c s="995" r="AT81"/>
+      <c s="995" r="AU81"/>
+      <c s="995" r="AV81"/>
+      <c s="995" r="AW81"/>
+      <c s="995" r="AX81"/>
+      <c s="995" r="AY81"/>
+      <c s="995" r="AZ81"/>
+      <c s="995" r="BA81"/>
+      <c s="995" r="BB81"/>
+      <c s="995" r="BC81"/>
+      <c s="995" r="BD81"/>
+      <c s="995" r="BE81"/>
+      <c s="995" r="BF81"/>
+      <c s="995" r="BG81"/>
+      <c s="995" r="BH81"/>
+      <c s="995" r="BI81"/>
+      <c s="995" r="BJ81"/>
+      <c s="995" r="BK81"/>
+      <c s="995" r="BL81"/>
+      <c s="995" r="BM81"/>
+      <c s="995" r="BN81"/>
+      <c s="995" r="BO81"/>
+      <c s="995" r="BP81"/>
+      <c s="995" r="BQ81"/>
+      <c s="995" r="BR81"/>
+      <c s="995" r="BS81"/>
+      <c s="995" r="BT81"/>
+      <c s="995" r="BU81"/>
+      <c s="995" r="BV81"/>
+      <c s="995" r="BW81"/>
+      <c s="995" r="BX81"/>
+      <c s="995" r="BY81"/>
+      <c s="995" r="BZ81"/>
+      <c s="995" r="CA81"/>
+      <c s="995" r="CB81"/>
+      <c s="995" r="CC81"/>
+      <c s="995" r="CD81"/>
+      <c s="995" r="CE81"/>
+      <c s="995" r="CF81"/>
+      <c s="995" r="CG81"/>
+      <c s="995" r="CH81"/>
+      <c s="995" r="CI81"/>
+      <c s="995" r="CJ81"/>
+      <c s="995" r="CK81"/>
+      <c s="995" r="CL81"/>
+      <c s="995" r="CM81"/>
+      <c s="995" r="CN81"/>
+      <c s="995" r="CO81"/>
+      <c s="995" r="CP81"/>
+      <c s="995" r="CQ81"/>
+      <c s="995" r="CR81"/>
+      <c s="995" r="CS81"/>
+      <c s="995" r="CT81"/>
+      <c s="995" r="CU81"/>
+      <c s="995" r="CV81"/>
+      <c s="995" r="CW81"/>
+      <c s="995" r="CX81"/>
+      <c s="995" r="CY81"/>
+      <c s="995" r="CZ81"/>
+      <c s="995" r="DA81"/>
+      <c s="995" r="DB81"/>
+      <c s="995" r="DC81"/>
+      <c s="995" r="DD81"/>
+      <c s="995" r="DE81"/>
+      <c s="995" r="DF81"/>
+      <c s="995" r="DG81"/>
     </row>
-    <row r="82" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A82"/>
-      <c s="322" r="B82" t="str">
+    <row r="82" ht="24" customHeight="1">
+      <c s="995" r="A82"/>
+      <c s="1006" r="B82" t="str">
         <v>单位与正负</v>
       </c>
-      <c s="331" r="C82"/>
-      <c s="332" r="D82" t="str">
+      <c s="995" r="C82"/>
+      <c s="1001" r="D82" t="str">
         <v>销量填整数台数，MSRP填正数，成本及费用填负数元/台。原表数字格式仅影响显示，实际数值精度保留。</v>
       </c>
-      <c s="332" r="E82"/>
-      <c s="333" r="F82"/>
-      <c s="332" r="G82"/>
-      <c s="332" r="H82"/>
-      <c s="333" r="I82"/>
-      <c s="332" r="J82"/>
-      <c s="332" r="K82"/>
-      <c s="333" r="L82"/>
-      <c s="332" r="M82"/>
-      <c s="332" r="N82"/>
-      <c s="333" r="O82"/>
-      <c s="332" r="P82"/>
-      <c s="332" r="Q82"/>
-      <c s="334" r="R82"/>
-      <c s="332" r="S82"/>
-      <c s="332" r="T82"/>
-      <c s="324" r="U82"/>
-      <c s="332" r="V82"/>
-      <c s="332" r="W82"/>
-      <c s="333" r="X82"/>
-      <c s="332" r="Y82"/>
-      <c s="332" r="Z82"/>
-      <c s="333" r="AA82"/>
-      <c s="332" r="AB82"/>
-      <c s="332" r="AC82"/>
-      <c s="333" r="AD82"/>
-      <c s="332" r="AE82"/>
-      <c s="332" r="AF82"/>
-      <c s="333" r="AG82"/>
-      <c s="332" r="AH82"/>
-      <c s="332" r="AI82"/>
-      <c s="334" r="AJ82"/>
-      <c s="332" r="AK82"/>
-      <c s="332" r="AL82"/>
-      <c s="324" r="AM82"/>
-      <c s="332" r="AN82"/>
-      <c s="332" r="AO82"/>
-      <c s="333" r="AP82"/>
-      <c s="332" r="AQ82"/>
-      <c s="332" r="AR82"/>
-      <c s="333" r="AS82"/>
-      <c s="332" r="AT82"/>
-      <c s="332" r="AU82"/>
-      <c s="333" r="AV82"/>
-      <c s="332" r="AW82"/>
-      <c s="332" r="AX82"/>
-      <c s="333" r="AY82"/>
-      <c s="332" r="AZ82"/>
-      <c s="332" r="BA82"/>
-      <c s="334" r="BB82"/>
-      <c s="332" r="BC82"/>
-      <c s="332" r="BD82"/>
-      <c s="324" r="BE82"/>
-      <c s="332" r="BF82"/>
-      <c s="332" r="BG82"/>
-      <c s="333" r="BH82"/>
-      <c s="332" r="BI82"/>
-      <c s="332" r="BJ82"/>
-      <c s="333" r="BK82"/>
-      <c s="332" r="BL82"/>
-      <c s="332" r="BM82"/>
-      <c s="333" r="BN82"/>
-      <c s="332" r="BO82"/>
-      <c s="332" r="BP82"/>
-      <c s="333" r="BQ82"/>
-      <c s="332" r="BR82"/>
-      <c s="332" r="BS82"/>
-      <c s="334" r="BT82"/>
-      <c s="332" r="BU82"/>
-      <c s="332" r="BV82"/>
-      <c s="324" r="BW82"/>
-      <c s="332" r="BX82"/>
-      <c s="332" r="BY82"/>
-      <c s="333" r="BZ82"/>
-      <c s="332" r="CA82"/>
-      <c s="332" r="CB82"/>
-      <c s="333" r="CC82"/>
-      <c s="332" r="CD82"/>
-      <c s="332" r="CE82"/>
-      <c s="333" r="CF82"/>
-      <c s="332" r="CG82"/>
-      <c s="332" r="CH82"/>
-      <c s="333" r="CI82"/>
-      <c s="332" r="CJ82"/>
-      <c s="332" r="CK82"/>
-      <c s="334" r="CL82"/>
-      <c s="332" r="CM82"/>
-      <c s="332" r="CN82"/>
-      <c s="325" r="CO82"/>
-      <c s="332" r="CP82"/>
-      <c s="332" r="CQ82"/>
-      <c s="326" r="CR82"/>
-      <c s="332" r="CS82"/>
-      <c s="332" r="CT82"/>
-      <c s="326" r="CU82"/>
-      <c s="332" r="CV82"/>
-      <c s="332" r="CW82"/>
-      <c s="326" r="CX82"/>
-      <c s="332" r="CY82"/>
-      <c s="332" r="CZ82"/>
-      <c s="326" r="DA82"/>
-      <c s="332" r="DB82"/>
-      <c s="332" r="DC82"/>
-      <c s="326" r="DD82"/>
-      <c s="332" r="DE82"/>
-      <c s="332" r="DF82"/>
-      <c s="335" r="DG82"/>
+      <c s="1001" r="E82"/>
+      <c s="1001" r="F82"/>
+      <c s="1001" r="G82"/>
+      <c s="1001" r="H82"/>
+      <c s="1001" r="I82"/>
+      <c s="1001" r="J82"/>
+      <c s="1001" r="K82"/>
+      <c s="1001" r="L82"/>
+      <c s="1001" r="M82"/>
+      <c s="1001" r="N82"/>
+      <c s="1001" r="O82"/>
+      <c s="1001" r="P82"/>
+      <c s="1001" r="Q82"/>
+      <c s="1001" r="R82"/>
+      <c s="1001" r="S82"/>
+      <c s="1001" r="T82"/>
+      <c s="995" r="U82"/>
+      <c s="995" r="V82"/>
+      <c s="995" r="W82"/>
+      <c s="995" r="X82"/>
+      <c s="995" r="Y82"/>
+      <c s="995" r="Z82"/>
+      <c s="995" r="AA82"/>
+      <c s="995" r="AB82"/>
+      <c s="995" r="AC82"/>
+      <c s="995" r="AD82"/>
+      <c s="995" r="AE82"/>
+      <c s="995" r="AF82"/>
+      <c s="995" r="AG82"/>
+      <c s="995" r="AH82"/>
+      <c s="995" r="AI82"/>
+      <c s="995" r="AJ82"/>
+      <c s="995" r="AK82"/>
+      <c s="995" r="AL82"/>
+      <c s="995" r="AM82"/>
+      <c s="995" r="AN82"/>
+      <c s="995" r="AO82"/>
+      <c s="995" r="AP82"/>
+      <c s="995" r="AQ82"/>
+      <c s="995" r="AR82"/>
+      <c s="995" r="AS82"/>
+      <c s="995" r="AT82"/>
+      <c s="995" r="AU82"/>
+      <c s="995" r="AV82"/>
+      <c s="995" r="AW82"/>
+      <c s="995" r="AX82"/>
+      <c s="995" r="AY82"/>
+      <c s="995" r="AZ82"/>
+      <c s="995" r="BA82"/>
+      <c s="995" r="BB82"/>
+      <c s="995" r="BC82"/>
+      <c s="995" r="BD82"/>
+      <c s="995" r="BE82"/>
+      <c s="995" r="BF82"/>
+      <c s="995" r="BG82"/>
+      <c s="995" r="BH82"/>
+      <c s="995" r="BI82"/>
+      <c s="995" r="BJ82"/>
+      <c s="995" r="BK82"/>
+      <c s="995" r="BL82"/>
+      <c s="995" r="BM82"/>
+      <c s="995" r="BN82"/>
+      <c s="995" r="BO82"/>
+      <c s="995" r="BP82"/>
+      <c s="995" r="BQ82"/>
+      <c s="995" r="BR82"/>
+      <c s="995" r="BS82"/>
+      <c s="995" r="BT82"/>
+      <c s="995" r="BU82"/>
+      <c s="995" r="BV82"/>
+      <c s="995" r="BW82"/>
+      <c s="995" r="BX82"/>
+      <c s="995" r="BY82"/>
+      <c s="995" r="BZ82"/>
+      <c s="995" r="CA82"/>
+      <c s="995" r="CB82"/>
+      <c s="995" r="CC82"/>
+      <c s="995" r="CD82"/>
+      <c s="995" r="CE82"/>
+      <c s="995" r="CF82"/>
+      <c s="995" r="CG82"/>
+      <c s="995" r="CH82"/>
+      <c s="995" r="CI82"/>
+      <c s="995" r="CJ82"/>
+      <c s="995" r="CK82"/>
+      <c s="995" r="CL82"/>
+      <c s="995" r="CM82"/>
+      <c s="995" r="CN82"/>
+      <c s="995" r="CO82"/>
+      <c s="995" r="CP82"/>
+      <c s="995" r="CQ82"/>
+      <c s="995" r="CR82"/>
+      <c s="995" r="CS82"/>
+      <c s="995" r="CT82"/>
+      <c s="995" r="CU82"/>
+      <c s="995" r="CV82"/>
+      <c s="995" r="CW82"/>
+      <c s="995" r="CX82"/>
+      <c s="995" r="CY82"/>
+      <c s="995" r="CZ82"/>
+      <c s="995" r="DA82"/>
+      <c s="995" r="DB82"/>
+      <c s="995" r="DC82"/>
+      <c s="995" r="DD82"/>
+      <c s="995" r="DE82"/>
+      <c s="995" r="DF82"/>
+      <c s="995" r="DG82"/>
     </row>
-    <row r="83" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A83"/>
-      <c s="322" r="B83" t="str">
+    <row r="83" ht="24" customHeight="1">
+      <c s="995" r="A83"/>
+      <c s="1006" r="B83" t="str">
         <v>固定费用</v>
       </c>
-      <c s="331" r="C83"/>
-      <c s="332" r="D83" t="str">
+      <c s="995" r="C83"/>
+      <c s="1001" r="D83" t="str">
         <v>固定制造费用、研发分摊、固定销交服及集团分摊，填已经分摊到单车的金额；本表不随销量自动重新分摊。</v>
       </c>
-      <c s="332" r="E83"/>
-      <c s="333" r="F83"/>
-      <c s="332" r="G83"/>
-      <c s="332" r="H83"/>
-      <c s="333" r="I83"/>
-      <c s="332" r="J83"/>
-      <c s="332" r="K83"/>
-      <c s="333" r="L83"/>
-      <c s="332" r="M83"/>
-      <c s="332" r="N83"/>
-      <c s="333" r="O83"/>
-      <c s="332" r="P83"/>
-      <c s="332" r="Q83"/>
-      <c s="334" r="R83"/>
-      <c s="332" r="S83"/>
-      <c s="332" r="T83"/>
-      <c s="324" r="U83"/>
-      <c s="332" r="V83"/>
-      <c s="332" r="W83"/>
-      <c s="333" r="X83"/>
-      <c s="332" r="Y83"/>
-      <c s="332" r="Z83"/>
-      <c s="333" r="AA83"/>
-      <c s="332" r="AB83"/>
-      <c s="332" r="AC83"/>
-      <c s="333" r="AD83"/>
-      <c s="332" r="AE83"/>
-      <c s="332" r="AF83"/>
-      <c s="333" r="AG83"/>
-      <c s="332" r="AH83"/>
-      <c s="332" r="AI83"/>
-      <c s="334" r="AJ83"/>
-      <c s="332" r="AK83"/>
-      <c s="332" r="AL83"/>
-      <c s="324" r="AM83"/>
-      <c s="332" r="AN83"/>
-      <c s="332" r="AO83"/>
-      <c s="333" r="AP83"/>
-      <c s="332" r="AQ83"/>
-      <c s="332" r="AR83"/>
-      <c s="333" r="AS83"/>
-      <c s="332" r="AT83"/>
-      <c s="332" r="AU83"/>
-      <c s="333" r="AV83"/>
-      <c s="332" r="AW83"/>
-      <c s="332" r="AX83"/>
-      <c s="333" r="AY83"/>
-      <c s="332" r="AZ83"/>
-      <c s="332" r="BA83"/>
-      <c s="334" r="BB83"/>
-      <c s="332" r="BC83"/>
-      <c s="332" r="BD83"/>
-      <c s="324" r="BE83"/>
-      <c s="332" r="BF83"/>
-      <c s="332" r="BG83"/>
-      <c s="333" r="BH83"/>
-      <c s="332" r="BI83"/>
-      <c s="332" r="BJ83"/>
-      <c s="333" r="BK83"/>
-      <c s="332" r="BL83"/>
-      <c s="332" r="BM83"/>
-      <c s="333" r="BN83"/>
-      <c s="332" r="BO83"/>
-      <c s="332" r="BP83"/>
-      <c s="333" r="BQ83"/>
-      <c s="332" r="BR83"/>
-      <c s="332" r="BS83"/>
-      <c s="334" r="BT83"/>
-      <c s="332" r="BU83"/>
-      <c s="332" r="BV83"/>
-      <c s="324" r="BW83"/>
-      <c s="332" r="BX83"/>
-      <c s="332" r="BY83"/>
-      <c s="333" r="BZ83"/>
-      <c s="332" r="CA83"/>
-      <c s="332" r="CB83"/>
-      <c s="333" r="CC83"/>
-      <c s="332" r="CD83"/>
-      <c s="332" r="CE83"/>
-      <c s="333" r="CF83"/>
-      <c s="332" r="CG83"/>
-      <c s="332" r="CH83"/>
-      <c s="333" r="CI83"/>
-      <c s="332" r="CJ83"/>
-      <c s="332" r="CK83"/>
-      <c s="334" r="CL83"/>
-      <c s="332" r="CM83"/>
-      <c s="332" r="CN83"/>
-      <c s="325" r="CO83"/>
-      <c s="332" r="CP83"/>
-      <c s="332" r="CQ83"/>
-      <c s="326" r="CR83"/>
-      <c s="332" r="CS83"/>
-      <c s="332" r="CT83"/>
-      <c s="326" r="CU83"/>
-      <c s="332" r="CV83"/>
-      <c s="332" r="CW83"/>
-      <c s="326" r="CX83"/>
-      <c s="332" r="CY83"/>
-      <c s="332" r="CZ83"/>
-      <c s="326" r="DA83"/>
-      <c s="332" r="DB83"/>
-      <c s="332" r="DC83"/>
-      <c s="326" r="DD83"/>
-      <c s="332" r="DE83"/>
-      <c s="332" r="DF83"/>
-      <c s="335" r="DG83"/>
+      <c s="1001" r="E83"/>
+      <c s="1001" r="F83"/>
+      <c s="1001" r="G83"/>
+      <c s="1001" r="H83"/>
+      <c s="1001" r="I83"/>
+      <c s="1001" r="J83"/>
+      <c s="1001" r="K83"/>
+      <c s="1001" r="L83"/>
+      <c s="1001" r="M83"/>
+      <c s="1001" r="N83"/>
+      <c s="1001" r="O83"/>
+      <c s="1001" r="P83"/>
+      <c s="1001" r="Q83"/>
+      <c s="1001" r="R83"/>
+      <c s="1001" r="S83"/>
+      <c s="1001" r="T83"/>
+      <c s="995" r="U83"/>
+      <c s="995" r="V83"/>
+      <c s="995" r="W83"/>
+      <c s="995" r="X83"/>
+      <c s="995" r="Y83"/>
+      <c s="995" r="Z83"/>
+      <c s="995" r="AA83"/>
+      <c s="995" r="AB83"/>
+      <c s="995" r="AC83"/>
+      <c s="995" r="AD83"/>
+      <c s="995" r="AE83"/>
+      <c s="995" r="AF83"/>
+      <c s="995" r="AG83"/>
+      <c s="995" r="AH83"/>
+      <c s="995" r="AI83"/>
+      <c s="995" r="AJ83"/>
+      <c s="995" r="AK83"/>
+      <c s="995" r="AL83"/>
+      <c s="995" r="AM83"/>
+      <c s="995" r="AN83"/>
+      <c s="995" r="AO83"/>
+      <c s="995" r="AP83"/>
+      <c s="995" r="AQ83"/>
+      <c s="995" r="AR83"/>
+      <c s="995" r="AS83"/>
+      <c s="995" r="AT83"/>
+      <c s="995" r="AU83"/>
+      <c s="995" r="AV83"/>
+      <c s="995" r="AW83"/>
+      <c s="995" r="AX83"/>
+      <c s="995" r="AY83"/>
+      <c s="995" r="AZ83"/>
+      <c s="995" r="BA83"/>
+      <c s="995" r="BB83"/>
+      <c s="995" r="BC83"/>
+      <c s="995" r="BD83"/>
+      <c s="995" r="BE83"/>
+      <c s="995" r="BF83"/>
+      <c s="995" r="BG83"/>
+      <c s="995" r="BH83"/>
+      <c s="995" r="BI83"/>
+      <c s="995" r="BJ83"/>
+      <c s="995" r="BK83"/>
+      <c s="995" r="BL83"/>
+      <c s="995" r="BM83"/>
+      <c s="995" r="BN83"/>
+      <c s="995" r="BO83"/>
+      <c s="995" r="BP83"/>
+      <c s="995" r="BQ83"/>
+      <c s="995" r="BR83"/>
+      <c s="995" r="BS83"/>
+      <c s="995" r="BT83"/>
+      <c s="995" r="BU83"/>
+      <c s="995" r="BV83"/>
+      <c s="995" r="BW83"/>
+      <c s="995" r="BX83"/>
+      <c s="995" r="BY83"/>
+      <c s="995" r="BZ83"/>
+      <c s="995" r="CA83"/>
+      <c s="995" r="CB83"/>
+      <c s="995" r="CC83"/>
+      <c s="995" r="CD83"/>
+      <c s="995" r="CE83"/>
+      <c s="995" r="CF83"/>
+      <c s="995" r="CG83"/>
+      <c s="995" r="CH83"/>
+      <c s="995" r="CI83"/>
+      <c s="995" r="CJ83"/>
+      <c s="995" r="CK83"/>
+      <c s="995" r="CL83"/>
+      <c s="995" r="CM83"/>
+      <c s="995" r="CN83"/>
+      <c s="995" r="CO83"/>
+      <c s="995" r="CP83"/>
+      <c s="995" r="CQ83"/>
+      <c s="995" r="CR83"/>
+      <c s="995" r="CS83"/>
+      <c s="995" r="CT83"/>
+      <c s="995" r="CU83"/>
+      <c s="995" r="CV83"/>
+      <c s="995" r="CW83"/>
+      <c s="995" r="CX83"/>
+      <c s="995" r="CY83"/>
+      <c s="995" r="CZ83"/>
+      <c s="995" r="DA83"/>
+      <c s="995" r="DB83"/>
+      <c s="995" r="DC83"/>
+      <c s="995" r="DD83"/>
+      <c s="995" r="DE83"/>
+      <c s="995" r="DF83"/>
+      <c s="995" r="DG83"/>
     </row>
-    <row r="84" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A84"/>
-      <c s="322" r="B84" t="str">
+    <row r="84" ht="24" customHeight="1">
+      <c s="995" r="A84"/>
+      <c s="1006" r="B84" t="str">
         <v>汇总顺序</v>
       </c>
-      <c s="331" r="C84"/>
-      <c s="332" r="D84" t="str">
+      <c s="995" r="C84"/>
+      <c s="1001" r="D84" t="str">
         <v>收入抵减逐项相加；MSRP加VAT及抵减得到净收入，净收入加成本得到毛利，毛利加费用得到EBIT。集团分摊计入费用。</v>
       </c>
-      <c s="332" r="E84"/>
-      <c s="333" r="F84"/>
-      <c s="332" r="G84"/>
-      <c s="332" r="H84"/>
-      <c s="333" r="I84"/>
-      <c s="332" r="J84"/>
-      <c s="332" r="K84"/>
-      <c s="333" r="L84"/>
-      <c s="332" r="M84"/>
-      <c s="332" r="N84"/>
-      <c s="333" r="O84"/>
-      <c s="332" r="P84"/>
-      <c s="332" r="Q84"/>
-      <c s="334" r="R84"/>
-      <c s="332" r="S84"/>
-      <c s="332" r="T84"/>
-      <c s="324" r="U84"/>
-      <c s="332" r="V84"/>
-      <c s="332" r="W84"/>
-      <c s="333" r="X84"/>
-      <c s="332" r="Y84"/>
-      <c s="332" r="Z84"/>
-      <c s="333" r="AA84"/>
-      <c s="332" r="AB84"/>
-      <c s="332" r="AC84"/>
-      <c s="333" r="AD84"/>
-      <c s="332" r="AE84"/>
-      <c s="332" r="AF84"/>
-      <c s="333" r="AG84"/>
-      <c s="332" r="AH84"/>
-      <c s="332" r="AI84"/>
-      <c s="334" r="AJ84"/>
-      <c s="332" r="AK84"/>
-      <c s="332" r="AL84"/>
-      <c s="324" r="AM84"/>
-      <c s="332" r="AN84"/>
-      <c s="332" r="AO84"/>
-      <c s="333" r="AP84"/>
-      <c s="332" r="AQ84"/>
-      <c s="332" r="AR84"/>
-      <c s="333" r="AS84"/>
-      <c s="332" r="AT84"/>
-      <c s="332" r="AU84"/>
-      <c s="333" r="AV84"/>
-      <c s="332" r="AW84"/>
-      <c s="332" r="AX84"/>
-      <c s="333" r="AY84"/>
-      <c s="332" r="AZ84"/>
-      <c s="332" r="BA84"/>
-      <c s="334" r="BB84"/>
-      <c s="332" r="BC84"/>
-      <c s="332" r="BD84"/>
-      <c s="324" r="BE84"/>
-      <c s="332" r="BF84"/>
-      <c s="332" r="BG84"/>
-      <c s="333" r="BH84"/>
-      <c s="332" r="BI84"/>
-      <c s="332" r="BJ84"/>
-      <c s="333" r="BK84"/>
-      <c s="332" r="BL84"/>
-      <c s="332" r="BM84"/>
-      <c s="333" r="BN84"/>
-      <c s="332" r="BO84"/>
-      <c s="332" r="BP84"/>
-      <c s="333" r="BQ84"/>
-      <c s="332" r="BR84"/>
-      <c s="332" r="BS84"/>
-      <c s="334" r="BT84"/>
-      <c s="332" r="BU84"/>
-      <c s="332" r="BV84"/>
-      <c s="324" r="BW84"/>
-      <c s="332" r="BX84"/>
-      <c s="332" r="BY84"/>
-      <c s="333" r="BZ84"/>
-      <c s="332" r="CA84"/>
-      <c s="332" r="CB84"/>
-      <c s="333" r="CC84"/>
-      <c s="332" r="CD84"/>
-      <c s="332" r="CE84"/>
-      <c s="333" r="CF84"/>
-      <c s="332" r="CG84"/>
-      <c s="332" r="CH84"/>
-      <c s="333" r="CI84"/>
-      <c s="332" r="CJ84"/>
-      <c s="332" r="CK84"/>
-      <c s="334" r="CL84"/>
-      <c s="332" r="CM84"/>
-      <c s="332" r="CN84"/>
-      <c s="325" r="CO84"/>
-      <c s="332" r="CP84"/>
-      <c s="332" r="CQ84"/>
-      <c s="326" r="CR84"/>
-      <c s="332" r="CS84"/>
-      <c s="332" r="CT84"/>
-      <c s="326" r="CU84"/>
-      <c s="332" r="CV84"/>
-      <c s="332" r="CW84"/>
-      <c s="326" r="CX84"/>
-      <c s="332" r="CY84"/>
-      <c s="332" r="CZ84"/>
-      <c s="326" r="DA84"/>
-      <c s="332" r="DB84"/>
-      <c s="332" r="DC84"/>
-      <c s="326" r="DD84"/>
-      <c s="332" r="DE84"/>
-      <c s="332" r="DF84"/>
-      <c s="335" r="DG84"/>
+      <c s="1001" r="E84"/>
+      <c s="1001" r="F84"/>
+      <c s="1001" r="G84"/>
+      <c s="1001" r="H84"/>
+      <c s="1001" r="I84"/>
+      <c s="1001" r="J84"/>
+      <c s="1001" r="K84"/>
+      <c s="1001" r="L84"/>
+      <c s="1001" r="M84"/>
+      <c s="1001" r="N84"/>
+      <c s="1001" r="O84"/>
+      <c s="1001" r="P84"/>
+      <c s="1001" r="Q84"/>
+      <c s="1001" r="R84"/>
+      <c s="1001" r="S84"/>
+      <c s="1001" r="T84"/>
+      <c s="995" r="U84"/>
+      <c s="995" r="V84"/>
+      <c s="995" r="W84"/>
+      <c s="995" r="X84"/>
+      <c s="995" r="Y84"/>
+      <c s="995" r="Z84"/>
+      <c s="995" r="AA84"/>
+      <c s="995" r="AB84"/>
+      <c s="995" r="AC84"/>
+      <c s="995" r="AD84"/>
+      <c s="995" r="AE84"/>
+      <c s="995" r="AF84"/>
+      <c s="995" r="AG84"/>
+      <c s="995" r="AH84"/>
+      <c s="995" r="AI84"/>
+      <c s="995" r="AJ84"/>
+      <c s="995" r="AK84"/>
+      <c s="995" r="AL84"/>
+      <c s="995" r="AM84"/>
+      <c s="995" r="AN84"/>
+      <c s="995" r="AO84"/>
+      <c s="995" r="AP84"/>
+      <c s="995" r="AQ84"/>
+      <c s="995" r="AR84"/>
+      <c s="995" r="AS84"/>
+      <c s="995" r="AT84"/>
+      <c s="995" r="AU84"/>
+      <c s="995" r="AV84"/>
+      <c s="995" r="AW84"/>
+      <c s="995" r="AX84"/>
+      <c s="995" r="AY84"/>
+      <c s="995" r="AZ84"/>
+      <c s="995" r="BA84"/>
+      <c s="995" r="BB84"/>
+      <c s="995" r="BC84"/>
+      <c s="995" r="BD84"/>
+      <c s="995" r="BE84"/>
+      <c s="995" r="BF84"/>
+      <c s="995" r="BG84"/>
+      <c s="995" r="BH84"/>
+      <c s="995" r="BI84"/>
+      <c s="995" r="BJ84"/>
+      <c s="995" r="BK84"/>
+      <c s="995" r="BL84"/>
+      <c s="995" r="BM84"/>
+      <c s="995" r="BN84"/>
+      <c s="995" r="BO84"/>
+      <c s="995" r="BP84"/>
+      <c s="995" r="BQ84"/>
+      <c s="995" r="BR84"/>
+      <c s="995" r="BS84"/>
+      <c s="995" r="BT84"/>
+      <c s="995" r="BU84"/>
+      <c s="995" r="BV84"/>
+      <c s="995" r="BW84"/>
+      <c s="995" r="BX84"/>
+      <c s="995" r="BY84"/>
+      <c s="995" r="BZ84"/>
+      <c s="995" r="CA84"/>
+      <c s="995" r="CB84"/>
+      <c s="995" r="CC84"/>
+      <c s="995" r="CD84"/>
+      <c s="995" r="CE84"/>
+      <c s="995" r="CF84"/>
+      <c s="995" r="CG84"/>
+      <c s="995" r="CH84"/>
+      <c s="995" r="CI84"/>
+      <c s="995" r="CJ84"/>
+      <c s="995" r="CK84"/>
+      <c s="995" r="CL84"/>
+      <c s="995" r="CM84"/>
+      <c s="995" r="CN84"/>
+      <c s="995" r="CO84"/>
+      <c s="995" r="CP84"/>
+      <c s="995" r="CQ84"/>
+      <c s="995" r="CR84"/>
+      <c s="995" r="CS84"/>
+      <c s="995" r="CT84"/>
+      <c s="995" r="CU84"/>
+      <c s="995" r="CV84"/>
+      <c s="995" r="CW84"/>
+      <c s="995" r="CX84"/>
+      <c s="995" r="CY84"/>
+      <c s="995" r="CZ84"/>
+      <c s="995" r="DA84"/>
+      <c s="995" r="DB84"/>
+      <c s="995" r="DC84"/>
+      <c s="995" r="DD84"/>
+      <c s="995" r="DE84"/>
+      <c s="995" r="DF84"/>
+      <c s="995" r="DG84"/>
     </row>
-    <row r="85" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A85"/>
-      <c s="322" r="B85" t="str">
+    <row r="85" ht="24" customHeight="1">
+      <c s="995" r="A85"/>
+      <c s="1006" r="B85" t="str">
         <v>BOM与调整</v>
       </c>
-      <c s="331" r="C85"/>
-      <c s="332" r="D85" t="str">
+      <c s="995" r="C85"/>
+      <c s="1001" r="D85" t="str">
         <v>BOM成本总额＝基准BOM成本＋赠送配置＋供应商模具分摊。三个子项分别填负数元/台，由总额计入成本总额。</v>
       </c>
-      <c s="332" r="E85"/>
-      <c s="333" r="F85"/>
-      <c s="332" r="G85"/>
-      <c s="332" r="H85"/>
-      <c s="333" r="I85"/>
-      <c s="332" r="J85"/>
-      <c s="332" r="K85"/>
-      <c s="333" r="L85"/>
-      <c s="332" r="M85"/>
-      <c s="332" r="N85"/>
-      <c s="333" r="O85"/>
-      <c s="332" r="P85"/>
-      <c s="332" r="Q85"/>
-      <c s="334" r="R85"/>
-      <c s="332" r="S85"/>
-      <c s="332" r="T85"/>
-      <c s="324" r="U85"/>
-      <c s="332" r="V85"/>
-      <c s="332" r="W85"/>
-      <c s="333" r="X85"/>
-      <c s="332" r="Y85"/>
-      <c s="332" r="Z85"/>
-      <c s="333" r="AA85"/>
-      <c s="332" r="AB85"/>
-      <c s="332" r="AC85"/>
-      <c s="333" r="AD85"/>
-      <c s="332" r="AE85"/>
-      <c s="332" r="AF85"/>
-      <c s="333" r="AG85"/>
-      <c s="332" r="AH85"/>
-      <c s="332" r="AI85"/>
-      <c s="334" r="AJ85"/>
-      <c s="332" r="AK85"/>
-      <c s="332" r="AL85"/>
-      <c s="324" r="AM85"/>
-      <c s="332" r="AN85"/>
-      <c s="332" r="AO85"/>
-      <c s="333" r="AP85"/>
-      <c s="332" r="AQ85"/>
-      <c s="332" r="AR85"/>
-      <c s="333" r="AS85"/>
-      <c s="332" r="AT85"/>
-      <c s="332" r="AU85"/>
-      <c s="333" r="AV85"/>
-      <c s="332" r="AW85"/>
-      <c s="332" r="AX85"/>
-      <c s="333" r="AY85"/>
-      <c s="332" r="AZ85"/>
-      <c s="332" r="BA85"/>
-      <c s="334" r="BB85"/>
-      <c s="332" r="BC85"/>
-      <c s="332" r="BD85"/>
-      <c s="324" r="BE85"/>
-      <c s="332" r="BF85"/>
-      <c s="332" r="BG85"/>
-      <c s="333" r="BH85"/>
-      <c s="332" r="BI85"/>
-      <c s="332" r="BJ85"/>
-      <c s="333" r="BK85"/>
-      <c s="332" r="BL85"/>
-      <c s="332" r="BM85"/>
-      <c s="333" r="BN85"/>
-      <c s="332" r="BO85"/>
-      <c s="332" r="BP85"/>
-      <c s="333" r="BQ85"/>
-      <c s="332" r="BR85"/>
-      <c s="332" r="BS85"/>
-      <c s="334" r="BT85"/>
-      <c s="332" r="BU85"/>
-      <c s="332" r="BV85"/>
-      <c s="324" r="BW85"/>
-      <c s="332" r="BX85"/>
-      <c s="332" r="BY85"/>
-      <c s="333" r="BZ85"/>
-      <c s="332" r="CA85"/>
-      <c s="332" r="CB85"/>
-      <c s="333" r="CC85"/>
-      <c s="332" r="CD85"/>
-      <c s="332" r="CE85"/>
-      <c s="333" r="CF85"/>
-      <c s="332" r="CG85"/>
-      <c s="332" r="CH85"/>
-      <c s="333" r="CI85"/>
-      <c s="332" r="CJ85"/>
-      <c s="332" r="CK85"/>
-      <c s="334" r="CL85"/>
-      <c s="332" r="CM85"/>
-      <c s="332" r="CN85"/>
-      <c s="325" r="CO85"/>
-      <c s="332" r="CP85"/>
-      <c s="332" r="CQ85"/>
-      <c s="326" r="CR85"/>
-      <c s="332" r="CS85"/>
-      <c s="332" r="CT85"/>
-      <c s="326" r="CU85"/>
-      <c s="332" r="CV85"/>
-      <c s="332" r="CW85"/>
-      <c s="326" r="CX85"/>
-      <c s="332" r="CY85"/>
-      <c s="332" r="CZ85"/>
-      <c s="326" r="DA85"/>
-      <c s="332" r="DB85"/>
-      <c s="332" r="DC85"/>
-      <c s="326" r="DD85"/>
-      <c s="332" r="DE85"/>
-      <c s="332" r="DF85"/>
-      <c s="335" r="DG85"/>
+      <c s="1001" r="E85"/>
+      <c s="1001" r="F85"/>
+      <c s="1001" r="G85"/>
+      <c s="1001" r="H85"/>
+      <c s="1001" r="I85"/>
+      <c s="1001" r="J85"/>
+      <c s="1001" r="K85"/>
+      <c s="1001" r="L85"/>
+      <c s="1001" r="M85"/>
+      <c s="1001" r="N85"/>
+      <c s="1001" r="O85"/>
+      <c s="1001" r="P85"/>
+      <c s="1001" r="Q85"/>
+      <c s="1001" r="R85"/>
+      <c s="1001" r="S85"/>
+      <c s="1001" r="T85"/>
+      <c s="995" r="U85"/>
+      <c s="995" r="V85"/>
+      <c s="995" r="W85"/>
+      <c s="995" r="X85"/>
+      <c s="995" r="Y85"/>
+      <c s="995" r="Z85"/>
+      <c s="995" r="AA85"/>
+      <c s="995" r="AB85"/>
+      <c s="995" r="AC85"/>
+      <c s="995" r="AD85"/>
+      <c s="995" r="AE85"/>
+      <c s="995" r="AF85"/>
+      <c s="995" r="AG85"/>
+      <c s="995" r="AH85"/>
+      <c s="995" r="AI85"/>
+      <c s="995" r="AJ85"/>
+      <c s="995" r="AK85"/>
+      <c s="995" r="AL85"/>
+      <c s="995" r="AM85"/>
+      <c s="995" r="AN85"/>
+      <c s="995" r="AO85"/>
+      <c s="995" r="AP85"/>
+      <c s="995" r="AQ85"/>
+      <c s="995" r="AR85"/>
+      <c s="995" r="AS85"/>
+      <c s="995" r="AT85"/>
+      <c s="995" r="AU85"/>
+      <c s="995" r="AV85"/>
+      <c s="995" r="AW85"/>
+      <c s="995" r="AX85"/>
+      <c s="995" r="AY85"/>
+      <c s="995" r="AZ85"/>
+      <c s="995" r="BA85"/>
+      <c s="995" r="BB85"/>
+      <c s="995" r="BC85"/>
+      <c s="995" r="BD85"/>
+      <c s="995" r="BE85"/>
+      <c s="995" r="BF85"/>
+      <c s="995" r="BG85"/>
+      <c s="995" r="BH85"/>
+      <c s="995" r="BI85"/>
+      <c s="995" r="BJ85"/>
+      <c s="995" r="BK85"/>
+      <c s="995" r="BL85"/>
+      <c s="995" r="BM85"/>
+      <c s="995" r="BN85"/>
+      <c s="995" r="BO85"/>
+      <c s="995" r="BP85"/>
+      <c s="995" r="BQ85"/>
+      <c s="995" r="BR85"/>
+      <c s="995" r="BS85"/>
+      <c s="995" r="BT85"/>
+      <c s="995" r="BU85"/>
+      <c s="995" r="BV85"/>
+      <c s="995" r="BW85"/>
+      <c s="995" r="BX85"/>
+      <c s="995" r="BY85"/>
+      <c s="995" r="BZ85"/>
+      <c s="995" r="CA85"/>
+      <c s="995" r="CB85"/>
+      <c s="995" r="CC85"/>
+      <c s="995" r="CD85"/>
+      <c s="995" r="CE85"/>
+      <c s="995" r="CF85"/>
+      <c s="995" r="CG85"/>
+      <c s="995" r="CH85"/>
+      <c s="995" r="CI85"/>
+      <c s="995" r="CJ85"/>
+      <c s="995" r="CK85"/>
+      <c s="995" r="CL85"/>
+      <c s="995" r="CM85"/>
+      <c s="995" r="CN85"/>
+      <c s="995" r="CO85"/>
+      <c s="995" r="CP85"/>
+      <c s="995" r="CQ85"/>
+      <c s="995" r="CR85"/>
+      <c s="995" r="CS85"/>
+      <c s="995" r="CT85"/>
+      <c s="995" r="CU85"/>
+      <c s="995" r="CV85"/>
+      <c s="995" r="CW85"/>
+      <c s="995" r="CX85"/>
+      <c s="995" r="CY85"/>
+      <c s="995" r="CZ85"/>
+      <c s="995" r="DA85"/>
+      <c s="995" r="DB85"/>
+      <c s="995" r="DC85"/>
+      <c s="995" r="DD85"/>
+      <c s="995" r="DE85"/>
+      <c s="995" r="DF85"/>
+      <c s="995" r="DG85"/>
     </row>
-    <row r="86" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A86"/>
-      <c s="322" r="B86" t="str">
+    <row r="86" ht="24" customHeight="1">
+      <c s="995" r="A86"/>
+      <c s="1006" r="B86" t="str">
         <v>税费口径</v>
       </c>
-      <c s="331" r="C86"/>
-      <c s="332" r="D86" t="str">
+      <c s="995" r="C86"/>
+      <c s="1001" r="D86" t="str">
         <v>VAT按含税MSRP价内剔除；消费税按净收入计提；关税按所填计税基数乘税率，税率为0时可不填基数。</v>
       </c>
-      <c s="332" r="E86"/>
-      <c s="333" r="F86"/>
-      <c s="332" r="G86"/>
-      <c s="332" r="H86"/>
-      <c s="333" r="I86"/>
-      <c s="332" r="J86"/>
-      <c s="332" r="K86"/>
-      <c s="333" r="L86"/>
-      <c s="332" r="M86"/>
-      <c s="332" r="N86"/>
-      <c s="333" r="O86"/>
-      <c s="332" r="P86"/>
-      <c s="332" r="Q86"/>
-      <c s="334" r="R86"/>
-      <c s="332" r="S86"/>
-      <c s="332" r="T86"/>
-      <c s="324" r="U86"/>
-      <c s="332" r="V86"/>
-      <c s="332" r="W86"/>
-      <c s="333" r="X86"/>
-      <c s="332" r="Y86"/>
-      <c s="332" r="Z86"/>
-      <c s="333" r="AA86"/>
-      <c s="332" r="AB86"/>
-      <c s="332" r="AC86"/>
-      <c s="333" r="AD86"/>
-      <c s="332" r="AE86"/>
-      <c s="332" r="AF86"/>
-      <c s="333" r="AG86"/>
-      <c s="332" r="AH86"/>
-      <c s="332" r="AI86"/>
-      <c s="334" r="AJ86"/>
-      <c s="332" r="AK86"/>
-      <c s="332" r="AL86"/>
-      <c s="324" r="AM86"/>
-      <c s="332" r="AN86"/>
-      <c s="332" r="AO86"/>
-      <c s="333" r="AP86"/>
-      <c s="332" r="AQ86"/>
-      <c s="332" r="AR86"/>
-      <c s="333" r="AS86"/>
-      <c s="332" r="AT86"/>
-      <c s="332" r="AU86"/>
-      <c s="333" r="AV86"/>
-      <c s="332" r="AW86"/>
-      <c s="332" r="AX86"/>
-      <c s="333" r="AY86"/>
-      <c s="332" r="AZ86"/>
-      <c s="332" r="BA86"/>
-      <c s="334" r="BB86"/>
-      <c s="332" r="BC86"/>
-      <c s="332" r="BD86"/>
-      <c s="324" r="BE86"/>
-      <c s="332" r="BF86"/>
-      <c s="332" r="BG86"/>
-      <c s="333" r="BH86"/>
-      <c s="332" r="BI86"/>
-      <c s="332" r="BJ86"/>
-      <c s="333" r="BK86"/>
-      <c s="332" r="BL86"/>
-      <c s="332" r="BM86"/>
-      <c s="333" r="BN86"/>
-      <c s="332" r="BO86"/>
-      <c s="332" r="BP86"/>
-      <c s="333" r="BQ86"/>
-      <c s="332" r="BR86"/>
-      <c s="332" r="BS86"/>
-      <c s="334" r="BT86"/>
-      <c s="332" r="BU86"/>
-      <c s="332" r="BV86"/>
-      <c s="324" r="BW86"/>
-      <c s="332" r="BX86"/>
-      <c s="332" r="BY86"/>
-      <c s="333" r="BZ86"/>
-      <c s="332" r="CA86"/>
-      <c s="332" r="CB86"/>
-      <c s="333" r="CC86"/>
-      <c s="332" r="CD86"/>
-      <c s="332" r="CE86"/>
-      <c s="333" r="CF86"/>
-      <c s="332" r="CG86"/>
-      <c s="332" r="CH86"/>
-      <c s="333" r="CI86"/>
-      <c s="332" r="CJ86"/>
-      <c s="332" r="CK86"/>
-      <c s="334" r="CL86"/>
-      <c s="332" r="CM86"/>
-      <c s="332" r="CN86"/>
-      <c s="325" r="CO86"/>
-      <c s="332" r="CP86"/>
-      <c s="332" r="CQ86"/>
-      <c s="326" r="CR86"/>
-      <c s="332" r="CS86"/>
-      <c s="332" r="CT86"/>
-      <c s="326" r="CU86"/>
-      <c s="332" r="CV86"/>
-      <c s="332" r="CW86"/>
-      <c s="326" r="CX86"/>
-      <c s="332" r="CY86"/>
-      <c s="332" r="CZ86"/>
-      <c s="326" r="DA86"/>
-      <c s="332" r="DB86"/>
-      <c s="332" r="DC86"/>
-      <c s="326" r="DD86"/>
-      <c s="332" r="DE86"/>
-      <c s="332" r="DF86"/>
-      <c s="335" r="DG86"/>
+      <c s="1001" r="E86"/>
+      <c s="1001" r="F86"/>
+      <c s="1001" r="G86"/>
+      <c s="1001" r="H86"/>
+      <c s="1001" r="I86"/>
+      <c s="1001" r="J86"/>
+      <c s="1001" r="K86"/>
+      <c s="1001" r="L86"/>
+      <c s="1001" r="M86"/>
+      <c s="1001" r="N86"/>
+      <c s="1001" r="O86"/>
+      <c s="1001" r="P86"/>
+      <c s="1001" r="Q86"/>
+      <c s="1001" r="R86"/>
+      <c s="1001" r="S86"/>
+      <c s="1001" r="T86"/>
+      <c s="995" r="U86"/>
+      <c s="995" r="V86"/>
+      <c s="995" r="W86"/>
+      <c s="995" r="X86"/>
+      <c s="995" r="Y86"/>
+      <c s="995" r="Z86"/>
+      <c s="995" r="AA86"/>
+      <c s="995" r="AB86"/>
+      <c s="995" r="AC86"/>
+      <c s="995" r="AD86"/>
+      <c s="995" r="AE86"/>
+      <c s="995" r="AF86"/>
+      <c s="995" r="AG86"/>
+      <c s="995" r="AH86"/>
+      <c s="995" r="AI86"/>
+      <c s="995" r="AJ86"/>
+      <c s="995" r="AK86"/>
+      <c s="995" r="AL86"/>
+      <c s="995" r="AM86"/>
+      <c s="995" r="AN86"/>
+      <c s="995" r="AO86"/>
+      <c s="995" r="AP86"/>
+      <c s="995" r="AQ86"/>
+      <c s="995" r="AR86"/>
+      <c s="995" r="AS86"/>
+      <c s="995" r="AT86"/>
+      <c s="995" r="AU86"/>
+      <c s="995" r="AV86"/>
+      <c s="995" r="AW86"/>
+      <c s="995" r="AX86"/>
+      <c s="995" r="AY86"/>
+      <c s="995" r="AZ86"/>
+      <c s="995" r="BA86"/>
+      <c s="995" r="BB86"/>
+      <c s="995" r="BC86"/>
+      <c s="995" r="BD86"/>
+      <c s="995" r="BE86"/>
+      <c s="995" r="BF86"/>
+      <c s="995" r="BG86"/>
+      <c s="995" r="BH86"/>
+      <c s="995" r="BI86"/>
+      <c s="995" r="BJ86"/>
+      <c s="995" r="BK86"/>
+      <c s="995" r="BL86"/>
+      <c s="995" r="BM86"/>
+      <c s="995" r="BN86"/>
+      <c s="995" r="BO86"/>
+      <c s="995" r="BP86"/>
+      <c s="995" r="BQ86"/>
+      <c s="995" r="BR86"/>
+      <c s="995" r="BS86"/>
+      <c s="995" r="BT86"/>
+      <c s="995" r="BU86"/>
+      <c s="995" r="BV86"/>
+      <c s="995" r="BW86"/>
+      <c s="995" r="BX86"/>
+      <c s="995" r="BY86"/>
+      <c s="995" r="BZ86"/>
+      <c s="995" r="CA86"/>
+      <c s="995" r="CB86"/>
+      <c s="995" r="CC86"/>
+      <c s="995" r="CD86"/>
+      <c s="995" r="CE86"/>
+      <c s="995" r="CF86"/>
+      <c s="995" r="CG86"/>
+      <c s="995" r="CH86"/>
+      <c s="995" r="CI86"/>
+      <c s="995" r="CJ86"/>
+      <c s="995" r="CK86"/>
+      <c s="995" r="CL86"/>
+      <c s="995" r="CM86"/>
+      <c s="995" r="CN86"/>
+      <c s="995" r="CO86"/>
+      <c s="995" r="CP86"/>
+      <c s="995" r="CQ86"/>
+      <c s="995" r="CR86"/>
+      <c s="995" r="CS86"/>
+      <c s="995" r="CT86"/>
+      <c s="995" r="CU86"/>
+      <c s="995" r="CV86"/>
+      <c s="995" r="CW86"/>
+      <c s="995" r="CX86"/>
+      <c s="995" r="CY86"/>
+      <c s="995" r="CZ86"/>
+      <c s="995" r="DA86"/>
+      <c s="995" r="DB86"/>
+      <c s="995" r="DC86"/>
+      <c s="995" r="DD86"/>
+      <c s="995" r="DE86"/>
+      <c s="995" r="DF86"/>
+      <c s="995" r="DG86"/>
     </row>
-    <row r="87" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A87"/>
-      <c s="322" r="B87" t="str">
+    <row r="87" ht="24" customHeight="1">
+      <c s="995" r="A87"/>
+      <c s="1006" r="B87" t="str">
         <v>附加与质保</v>
       </c>
-      <c s="331" r="C87"/>
-      <c s="332" r="D87" t="str">
+      <c s="995" r="C87"/>
+      <c s="1001" r="D87" t="str">
         <v>城建附加沿用原测算模型，以BOM乘增值税率估算进项抵扣，增值税净额不低于0，再加消费税计算附加；质保按MSRP计提。</v>
       </c>
-      <c s="332" r="E87"/>
-      <c s="333" r="F87"/>
-      <c s="332" r="G87"/>
-      <c s="332" r="H87"/>
-      <c s="333" r="I87"/>
-      <c s="332" r="J87"/>
-      <c s="332" r="K87"/>
-      <c s="333" r="L87"/>
-      <c s="332" r="M87"/>
-      <c s="332" r="N87"/>
-      <c s="333" r="O87"/>
-      <c s="332" r="P87"/>
-      <c s="332" r="Q87"/>
-      <c s="334" r="R87"/>
-      <c s="332" r="S87"/>
-      <c s="332" r="T87"/>
-      <c s="324" r="U87"/>
-      <c s="332" r="V87"/>
-      <c s="332" r="W87"/>
-      <c s="333" r="X87"/>
-      <c s="332" r="Y87"/>
-      <c s="332" r="Z87"/>
-      <c s="333" r="AA87"/>
-      <c s="332" r="AB87"/>
-      <c s="332" r="AC87"/>
-      <c s="333" r="AD87"/>
-      <c s="332" r="AE87"/>
-      <c s="332" r="AF87"/>
-      <c s="333" r="AG87"/>
-      <c s="332" r="AH87"/>
-      <c s="332" r="AI87"/>
-      <c s="334" r="AJ87"/>
-      <c s="332" r="AK87"/>
-      <c s="332" r="AL87"/>
-      <c s="324" r="AM87"/>
-      <c s="332" r="AN87"/>
-      <c s="332" r="AO87"/>
-      <c s="333" r="AP87"/>
-      <c s="332" r="AQ87"/>
-      <c s="332" r="AR87"/>
-      <c s="333" r="AS87"/>
-      <c s="332" r="AT87"/>
-      <c s="332" r="AU87"/>
-      <c s="333" r="AV87"/>
-      <c s="332" r="AW87"/>
-      <c s="332" r="AX87"/>
-      <c s="333" r="AY87"/>
-      <c s="332" r="AZ87"/>
-      <c s="332" r="BA87"/>
-      <c s="334" r="BB87"/>
-      <c s="332" r="BC87"/>
-      <c s="332" r="BD87"/>
-      <c s="324" r="BE87"/>
-      <c s="332" r="BF87"/>
-      <c s="332" r="BG87"/>
-      <c s="333" r="BH87"/>
-      <c s="332" r="BI87"/>
-      <c s="332" r="BJ87"/>
-      <c s="333" r="BK87"/>
-      <c s="332" r="BL87"/>
-      <c s="332" r="BM87"/>
-      <c s="333" r="BN87"/>
-      <c s="332" r="BO87"/>
-      <c s="332" r="BP87"/>
-      <c s="333" r="BQ87"/>
-      <c s="332" r="BR87"/>
-      <c s="332" r="BS87"/>
-      <c s="334" r="BT87"/>
-      <c s="332" r="BU87"/>
-      <c s="332" r="BV87"/>
-      <c s="324" r="BW87"/>
-      <c s="332" r="BX87"/>
-      <c s="332" r="BY87"/>
-      <c s="333" r="BZ87"/>
-      <c s="332" r="CA87"/>
-      <c s="332" r="CB87"/>
-      <c s="333" r="CC87"/>
-      <c s="332" r="CD87"/>
-      <c s="332" r="CE87"/>
-      <c s="333" r="CF87"/>
-      <c s="332" r="CG87"/>
-      <c s="332" r="CH87"/>
-      <c s="333" r="CI87"/>
-      <c s="332" r="CJ87"/>
-      <c s="332" r="CK87"/>
-      <c s="334" r="CL87"/>
-      <c s="332" r="CM87"/>
-      <c s="332" r="CN87"/>
-      <c s="325" r="CO87"/>
-      <c s="332" r="CP87"/>
-      <c s="332" r="CQ87"/>
-      <c s="326" r="CR87"/>
-      <c s="332" r="CS87"/>
-      <c s="332" r="CT87"/>
-      <c s="326" r="CU87"/>
-      <c s="332" r="CV87"/>
-      <c s="332" r="CW87"/>
-      <c s="326" r="CX87"/>
-      <c s="332" r="CY87"/>
-      <c s="332" r="CZ87"/>
-      <c s="326" r="DA87"/>
-      <c s="332" r="DB87"/>
-      <c s="332" r="DC87"/>
-      <c s="326" r="DD87"/>
-      <c s="332" r="DE87"/>
-      <c s="332" r="DF87"/>
-      <c s="335" r="DG87"/>
+      <c s="1001" r="E87"/>
+      <c s="1001" r="F87"/>
+      <c s="1001" r="G87"/>
+      <c s="1001" r="H87"/>
+      <c s="1001" r="I87"/>
+      <c s="1001" r="J87"/>
+      <c s="1001" r="K87"/>
+      <c s="1001" r="L87"/>
+      <c s="1001" r="M87"/>
+      <c s="1001" r="N87"/>
+      <c s="1001" r="O87"/>
+      <c s="1001" r="P87"/>
+      <c s="1001" r="Q87"/>
+      <c s="1001" r="R87"/>
+      <c s="1001" r="S87"/>
+      <c s="1001" r="T87"/>
+      <c s="995" r="U87"/>
+      <c s="995" r="V87"/>
+      <c s="995" r="W87"/>
+      <c s="995" r="X87"/>
+      <c s="995" r="Y87"/>
+      <c s="995" r="Z87"/>
+      <c s="995" r="AA87"/>
+      <c s="995" r="AB87"/>
+      <c s="995" r="AC87"/>
+      <c s="995" r="AD87"/>
+      <c s="995" r="AE87"/>
+      <c s="995" r="AF87"/>
+      <c s="995" r="AG87"/>
+      <c s="995" r="AH87"/>
+      <c s="995" r="AI87"/>
+      <c s="995" r="AJ87"/>
+      <c s="995" r="AK87"/>
+      <c s="995" r="AL87"/>
+      <c s="995" r="AM87"/>
+      <c s="995" r="AN87"/>
+      <c s="995" r="AO87"/>
+      <c s="995" r="AP87"/>
+      <c s="995" r="AQ87"/>
+      <c s="995" r="AR87"/>
+      <c s="995" r="AS87"/>
+      <c s="995" r="AT87"/>
+      <c s="995" r="AU87"/>
+      <c s="995" r="AV87"/>
+      <c s="995" r="AW87"/>
+      <c s="995" r="AX87"/>
+      <c s="995" r="AY87"/>
+      <c s="995" r="AZ87"/>
+      <c s="995" r="BA87"/>
+      <c s="995" r="BB87"/>
+      <c s="995" r="BC87"/>
+      <c s="995" r="BD87"/>
+      <c s="995" r="BE87"/>
+      <c s="995" r="BF87"/>
+      <c s="995" r="BG87"/>
+      <c s="995" r="BH87"/>
+      <c s="995" r="BI87"/>
+      <c s="995" r="BJ87"/>
+      <c s="995" r="BK87"/>
+      <c s="995" r="BL87"/>
+      <c s="995" r="BM87"/>
+      <c s="995" r="BN87"/>
+      <c s="995" r="BO87"/>
+      <c s="995" r="BP87"/>
+      <c s="995" r="BQ87"/>
+      <c s="995" r="BR87"/>
+      <c s="995" r="BS87"/>
+      <c s="995" r="BT87"/>
+      <c s="995" r="BU87"/>
+      <c s="995" r="BV87"/>
+      <c s="995" r="BW87"/>
+      <c s="995" r="BX87"/>
+      <c s="995" r="BY87"/>
+      <c s="995" r="BZ87"/>
+      <c s="995" r="CA87"/>
+      <c s="995" r="CB87"/>
+      <c s="995" r="CC87"/>
+      <c s="995" r="CD87"/>
+      <c s="995" r="CE87"/>
+      <c s="995" r="CF87"/>
+      <c s="995" r="CG87"/>
+      <c s="995" r="CH87"/>
+      <c s="995" r="CI87"/>
+      <c s="995" r="CJ87"/>
+      <c s="995" r="CK87"/>
+      <c s="995" r="CL87"/>
+      <c s="995" r="CM87"/>
+      <c s="995" r="CN87"/>
+      <c s="995" r="CO87"/>
+      <c s="995" r="CP87"/>
+      <c s="995" r="CQ87"/>
+      <c s="995" r="CR87"/>
+      <c s="995" r="CS87"/>
+      <c s="995" r="CT87"/>
+      <c s="995" r="CU87"/>
+      <c s="995" r="CV87"/>
+      <c s="995" r="CW87"/>
+      <c s="995" r="CX87"/>
+      <c s="995" r="CY87"/>
+      <c s="995" r="CZ87"/>
+      <c s="995" r="DA87"/>
+      <c s="995" r="DB87"/>
+      <c s="995" r="DC87"/>
+      <c s="995" r="DD87"/>
+      <c s="995" r="DE87"/>
+      <c s="995" r="DF87"/>
+      <c s="995" r="DG87"/>
     </row>
-    <row r="88" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A88"/>
-      <c s="322" r="B88" t="str">
+    <row r="88" ht="24" customHeight="1">
+      <c s="995" r="A88"/>
+      <c s="1006" r="B88" t="str">
         <v>参数与零值</v>
       </c>
-      <c s="331" r="C88"/>
-      <c s="332" r="D88" t="str">
+      <c s="995" r="C88"/>
+      <c s="1001" r="D88" t="str">
         <v>新增年度请复制完整年度组并修改SOP+n；保留车型与单车（元）标题。新增明细归入原上级，暂不增加调参联动。</v>
       </c>
-      <c s="332" r="E88"/>
-      <c s="333" r="F88"/>
-      <c s="332" r="G88"/>
-      <c s="332" r="H88"/>
-      <c s="333" r="I88"/>
-      <c s="332" r="J88"/>
-      <c s="332" r="K88"/>
-      <c s="333" r="L88"/>
-      <c s="332" r="M88"/>
-      <c s="332" r="N88"/>
-      <c s="333" r="O88"/>
-      <c s="332" r="P88"/>
-      <c s="332" r="Q88"/>
-      <c s="334" r="R88"/>
-      <c s="332" r="S88"/>
-      <c s="332" r="T88"/>
-      <c s="324" r="U88"/>
-      <c s="332" r="V88"/>
-      <c s="332" r="W88"/>
-      <c s="333" r="X88"/>
-      <c s="332" r="Y88"/>
-      <c s="332" r="Z88"/>
-      <c s="333" r="AA88"/>
-      <c s="332" r="AB88"/>
-      <c s="332" r="AC88"/>
-      <c s="333" r="AD88"/>
-      <c s="332" r="AE88"/>
-      <c s="332" r="AF88"/>
-      <c s="333" r="AG88"/>
-      <c s="332" r="AH88"/>
-      <c s="332" r="AI88"/>
-      <c s="334" r="AJ88"/>
-      <c s="332" r="AK88"/>
-      <c s="332" r="AL88"/>
-      <c s="324" r="AM88"/>
-      <c s="332" r="AN88"/>
-      <c s="332" r="AO88"/>
-      <c s="333" r="AP88"/>
-      <c s="332" r="AQ88"/>
-      <c s="332" r="AR88"/>
-      <c s="333" r="AS88"/>
-      <c s="332" r="AT88"/>
-      <c s="332" r="AU88"/>
-      <c s="333" r="AV88"/>
-      <c s="332" r="AW88"/>
-      <c s="332" r="AX88"/>
-      <c s="333" r="AY88"/>
-      <c s="332" r="AZ88"/>
-      <c s="332" r="BA88"/>
-      <c s="334" r="BB88"/>
-      <c s="332" r="BC88"/>
-      <c s="332" r="BD88"/>
-      <c s="324" r="BE88"/>
-      <c s="332" r="BF88"/>
-      <c s="332" r="BG88"/>
-      <c s="333" r="BH88"/>
-      <c s="332" r="BI88"/>
-      <c s="332" r="BJ88"/>
-      <c s="333" r="BK88"/>
-      <c s="332" r="BL88"/>
-      <c s="332" r="BM88"/>
-      <c s="333" r="BN88"/>
-      <c s="332" r="BO88"/>
-      <c s="332" r="BP88"/>
-      <c s="333" r="BQ88"/>
-      <c s="332" r="BR88"/>
-      <c s="332" r="BS88"/>
-      <c s="334" r="BT88"/>
-      <c s="332" r="BU88"/>
-      <c s="332" r="BV88"/>
-      <c s="324" r="BW88"/>
-      <c s="332" r="BX88"/>
-      <c s="332" r="BY88"/>
-      <c s="333" r="BZ88"/>
-      <c s="332" r="CA88"/>
-      <c s="332" r="CB88"/>
-      <c s="333" r="CC88"/>
-      <c s="332" r="CD88"/>
-      <c s="332" r="CE88"/>
-      <c s="333" r="CF88"/>
-      <c s="332" r="CG88"/>
-      <c s="332" r="CH88"/>
-      <c s="333" r="CI88"/>
-      <c s="332" r="CJ88"/>
-      <c s="332" r="CK88"/>
-      <c s="334" r="CL88"/>
-      <c s="332" r="CM88"/>
-      <c s="332" r="CN88"/>
-      <c s="325" r="CO88"/>
-      <c s="332" r="CP88"/>
-      <c s="332" r="CQ88"/>
-      <c s="326" r="CR88"/>
-      <c s="332" r="CS88"/>
-      <c s="332" r="CT88"/>
-      <c s="326" r="CU88"/>
-      <c s="332" r="CV88"/>
-      <c s="332" r="CW88"/>
-      <c s="326" r="CX88"/>
-      <c s="332" r="CY88"/>
-      <c s="332" r="CZ88"/>
-      <c s="326" r="DA88"/>
-      <c s="332" r="DB88"/>
-      <c s="332" r="DC88"/>
-      <c s="326" r="DD88"/>
-      <c s="332" r="DE88"/>
-      <c s="332" r="DF88"/>
-      <c s="335" r="DG88"/>
+      <c s="1001" r="E88"/>
+      <c s="1001" r="F88"/>
+      <c s="1001" r="G88"/>
+      <c s="1001" r="H88"/>
+      <c s="1001" r="I88"/>
+      <c s="1001" r="J88"/>
+      <c s="1001" r="K88"/>
+      <c s="1001" r="L88"/>
+      <c s="1001" r="M88"/>
+      <c s="1001" r="N88"/>
+      <c s="1001" r="O88"/>
+      <c s="1001" r="P88"/>
+      <c s="1001" r="Q88"/>
+      <c s="1001" r="R88"/>
+      <c s="1001" r="S88"/>
+      <c s="1001" r="T88"/>
+      <c s="995" r="U88"/>
+      <c s="995" r="V88"/>
+      <c s="995" r="W88"/>
+      <c s="995" r="X88"/>
+      <c s="995" r="Y88"/>
+      <c s="995" r="Z88"/>
+      <c s="995" r="AA88"/>
+      <c s="995" r="AB88"/>
+      <c s="995" r="AC88"/>
+      <c s="995" r="AD88"/>
+      <c s="995" r="AE88"/>
+      <c s="995" r="AF88"/>
+      <c s="995" r="AG88"/>
+      <c s="995" r="AH88"/>
+      <c s="995" r="AI88"/>
+      <c s="995" r="AJ88"/>
+      <c s="995" r="AK88"/>
+      <c s="995" r="AL88"/>
+      <c s="995" r="AM88"/>
+      <c s="995" r="AN88"/>
+      <c s="995" r="AO88"/>
+      <c s="995" r="AP88"/>
+      <c s="995" r="AQ88"/>
+      <c s="995" r="AR88"/>
+      <c s="995" r="AS88"/>
+      <c s="995" r="AT88"/>
+      <c s="995" r="AU88"/>
+      <c s="995" r="AV88"/>
+      <c s="995" r="AW88"/>
+      <c s="995" r="AX88"/>
+      <c s="995" r="AY88"/>
+      <c s="995" r="AZ88"/>
+      <c s="995" r="BA88"/>
+      <c s="995" r="BB88"/>
+      <c s="995" r="BC88"/>
+      <c s="995" r="BD88"/>
+      <c s="995" r="BE88"/>
+      <c s="995" r="BF88"/>
+      <c s="995" r="BG88"/>
+      <c s="995" r="BH88"/>
+      <c s="995" r="BI88"/>
+      <c s="995" r="BJ88"/>
+      <c s="995" r="BK88"/>
+      <c s="995" r="BL88"/>
+      <c s="995" r="BM88"/>
+      <c s="995" r="BN88"/>
+      <c s="995" r="BO88"/>
+      <c s="995" r="BP88"/>
+      <c s="995" r="BQ88"/>
+      <c s="995" r="BR88"/>
+      <c s="995" r="BS88"/>
+      <c s="995" r="BT88"/>
+      <c s="995" r="BU88"/>
+      <c s="995" r="BV88"/>
+      <c s="995" r="BW88"/>
+      <c s="995" r="BX88"/>
+      <c s="995" r="BY88"/>
+      <c s="995" r="BZ88"/>
+      <c s="995" r="CA88"/>
+      <c s="995" r="CB88"/>
+      <c s="995" r="CC88"/>
+      <c s="995" r="CD88"/>
+      <c s="995" r="CE88"/>
+      <c s="995" r="CF88"/>
+      <c s="995" r="CG88"/>
+      <c s="995" r="CH88"/>
+      <c s="995" r="CI88"/>
+      <c s="995" r="CJ88"/>
+      <c s="995" r="CK88"/>
+      <c s="995" r="CL88"/>
+      <c s="995" r="CM88"/>
+      <c s="995" r="CN88"/>
+      <c s="995" r="CO88"/>
+      <c s="995" r="CP88"/>
+      <c s="995" r="CQ88"/>
+      <c s="995" r="CR88"/>
+      <c s="995" r="CS88"/>
+      <c s="995" r="CT88"/>
+      <c s="995" r="CU88"/>
+      <c s="995" r="CV88"/>
+      <c s="995" r="CW88"/>
+      <c s="995" r="CX88"/>
+      <c s="995" r="CY88"/>
+      <c s="995" r="CZ88"/>
+      <c s="995" r="DA88"/>
+      <c s="995" r="DB88"/>
+      <c s="995" r="DC88"/>
+      <c s="995" r="DD88"/>
+      <c s="995" r="DE88"/>
+      <c s="995" r="DF88"/>
+      <c s="995" r="DG88"/>
     </row>
-    <row r="89" spans="1:111" ht="24" customHeight="1">
-      <c s="321" r="A89"/>
-      <c s="322" r="B89" t="str">
+    <row r="89" ht="24" customHeight="1">
+      <c s="995" r="A89"/>
+      <c s="1006" r="B89" t="str">
         <v>计算依据</v>
       </c>
-      <c s="331" r="C89"/>
-      <c s="332" r="D89" t="str">
+      <c s="995" r="C89"/>
+      <c s="1001" r="D89" t="str">
         <v>依据本模板的科目层级及《BC测算分析模板-线下.xlsx》已有计算关系；集团分摊沿用已确认的计入EBIT口径。</v>
       </c>
-      <c s="332" r="E89"/>
-      <c s="333" r="F89"/>
-      <c s="332" r="G89"/>
-      <c s="332" r="H89"/>
-      <c s="333" r="I89"/>
-      <c s="332" r="J89"/>
-      <c s="332" r="K89"/>
-      <c s="333" r="L89"/>
-      <c s="332" r="M89"/>
-      <c s="332" r="N89"/>
-      <c s="333" r="O89"/>
-      <c s="332" r="P89"/>
-      <c s="332" r="Q89"/>
-      <c s="334" r="R89"/>
-      <c s="332" r="S89"/>
-      <c s="332" r="T89"/>
-      <c s="324" r="U89"/>
-      <c s="332" r="V89"/>
-      <c s="332" r="W89"/>
-      <c s="333" r="X89"/>
-      <c s="332" r="Y89"/>
-      <c s="332" r="Z89"/>
-      <c s="333" r="AA89"/>
-      <c s="332" r="AB89"/>
-      <c s="332" r="AC89"/>
-      <c s="333" r="AD89"/>
-      <c s="332" r="AE89"/>
-      <c s="332" r="AF89"/>
-      <c s="333" r="AG89"/>
-      <c s="332" r="AH89"/>
-      <c s="332" r="AI89"/>
-      <c s="334" r="AJ89"/>
-      <c s="332" r="AK89"/>
-      <c s="332" r="AL89"/>
-      <c s="324" r="AM89"/>
-      <c s="332" r="AN89"/>
-      <c s="332" r="AO89"/>
-      <c s="333" r="AP89"/>
-      <c s="332" r="AQ89"/>
-      <c s="332" r="AR89"/>
-      <c s="333" r="AS89"/>
-      <c s="332" r="AT89"/>
-      <c s="332" r="AU89"/>
-      <c s="333" r="AV89"/>
-      <c s="332" r="AW89"/>
-      <c s="332" r="AX89"/>
-      <c s="333" r="AY89"/>
-      <c s="332" r="AZ89"/>
-      <c s="332" r="BA89"/>
-      <c s="334" r="BB89"/>
-      <c s="332" r="BC89"/>
-      <c s="332" r="BD89"/>
-      <c s="324" r="BE89"/>
-      <c s="332" r="BF89"/>
-      <c s="332" r="BG89"/>
-      <c s="333" r="BH89"/>
-      <c s="332" r="BI89"/>
-      <c s="332" r="BJ89"/>
-      <c s="333" r="BK89"/>
-      <c s="332" r="BL89"/>
-      <c s="332" r="BM89"/>
-      <c s="333" r="BN89"/>
-      <c s="332" r="BO89"/>
-      <c s="332" r="BP89"/>
-      <c s="333" r="BQ89"/>
-      <c s="332" r="BR89"/>
-      <c s="332" r="BS89"/>
-      <c s="334" r="BT89"/>
-      <c s="332" r="BU89"/>
-      <c s="332" r="BV89"/>
-      <c s="324" r="BW89"/>
-      <c s="332" r="BX89"/>
-      <c s="332" r="BY89"/>
-      <c s="333" r="BZ89"/>
-      <c s="332" r="CA89"/>
-      <c s="332" r="CB89"/>
-      <c s="333" r="CC89"/>
-      <c s="332" r="CD89"/>
-      <c s="332" r="CE89"/>
-      <c s="333" r="CF89"/>
-      <c s="332" r="CG89"/>
-      <c s="332" r="CH89"/>
-      <c s="333" r="CI89"/>
-      <c s="332" r="CJ89"/>
-      <c s="332" r="CK89"/>
-      <c s="334" r="CL89"/>
-      <c s="332" r="CM89"/>
-      <c s="332" r="CN89"/>
-      <c s="325" r="CO89"/>
-      <c s="332" r="CP89"/>
-      <c s="332" r="CQ89"/>
-      <c s="326" r="CR89"/>
-      <c s="332" r="CS89"/>
-      <c s="332" r="CT89"/>
-      <c s="326" r="CU89"/>
-      <c s="332" r="CV89"/>
-      <c s="332" r="CW89"/>
-      <c s="326" r="CX89"/>
-      <c s="332" r="CY89"/>
-      <c s="332" r="CZ89"/>
-      <c s="326" r="DA89"/>
-      <c s="332" r="DB89"/>
-      <c s="332" r="DC89"/>
-      <c s="326" r="DD89"/>
-      <c s="332" r="DE89"/>
-      <c s="332" r="DF89"/>
-      <c s="335" r="DG89"/>
+      <c s="1001" r="E89"/>
+      <c s="1001" r="F89"/>
+      <c s="1001" r="G89"/>
+      <c s="1001" r="H89"/>
+      <c s="1001" r="I89"/>
+      <c s="1001" r="J89"/>
+      <c s="1001" r="K89"/>
+      <c s="1001" r="L89"/>
+      <c s="1001" r="M89"/>
+      <c s="1001" r="N89"/>
+      <c s="1001" r="O89"/>
+      <c s="1001" r="P89"/>
+      <c s="1001" r="Q89"/>
+      <c s="1001" r="R89"/>
+      <c s="1001" r="S89"/>
+      <c s="1001" r="T89"/>
+      <c s="995" r="U89"/>
+      <c s="995" r="V89"/>
+      <c s="995" r="W89"/>
+      <c s="995" r="X89"/>
+      <c s="995" r="Y89"/>
+      <c s="995" r="Z89"/>
+      <c s="995" r="AA89"/>
+      <c s="995" r="AB89"/>
+      <c s="995" r="AC89"/>
+      <c s="995" r="AD89"/>
+      <c s="995" r="AE89"/>
+      <c s="995" r="AF89"/>
+      <c s="995" r="AG89"/>
+      <c s="995" r="AH89"/>
+      <c s="995" r="AI89"/>
+      <c s="995" r="AJ89"/>
+      <c s="995" r="AK89"/>
+      <c s="995" r="AL89"/>
+      <c s="995" r="AM89"/>
+      <c s="995" r="AN89"/>
+      <c s="995" r="AO89"/>
+      <c s="995" r="AP89"/>
+      <c s="995" r="AQ89"/>
+      <c s="995" r="AR89"/>
+      <c s="995" r="AS89"/>
+      <c s="995" r="AT89"/>
+      <c s="995" r="AU89"/>
+      <c s="995" r="AV89"/>
+      <c s="995" r="AW89"/>
+      <c s="995" r="AX89"/>
+      <c s="995" r="AY89"/>
+      <c s="995" r="AZ89"/>
+      <c s="995" r="BA89"/>
+      <c s="995" r="BB89"/>
+      <c s="995" r="BC89"/>
+      <c s="995" r="BD89"/>
+      <c s="995" r="BE89"/>
+      <c s="995" r="BF89"/>
+      <c s="995" r="BG89"/>
+      <c s="995" r="BH89"/>
+      <c s="995" r="BI89"/>
+      <c s="995" r="BJ89"/>
+      <c s="995" r="BK89"/>
+      <c s="995" r="BL89"/>
+      <c s="995" r="BM89"/>
+      <c s="995" r="BN89"/>
+      <c s="995" r="BO89"/>
+      <c s="995" r="BP89"/>
+      <c s="995" r="BQ89"/>
+      <c s="995" r="BR89"/>
+      <c s="995" r="BS89"/>
+      <c s="995" r="BT89"/>
+      <c s="995" r="BU89"/>
+      <c s="995" r="BV89"/>
+      <c s="995" r="BW89"/>
+      <c s="995" r="BX89"/>
+      <c s="995" r="BY89"/>
+      <c s="995" r="BZ89"/>
+      <c s="995" r="CA89"/>
+      <c s="995" r="CB89"/>
+      <c s="995" r="CC89"/>
+      <c s="995" r="CD89"/>
+      <c s="995" r="CE89"/>
+      <c s="995" r="CF89"/>
+      <c s="995" r="CG89"/>
+      <c s="995" r="CH89"/>
+      <c s="995" r="CI89"/>
+      <c s="995" r="CJ89"/>
+      <c s="995" r="CK89"/>
+      <c s="995" r="CL89"/>
+      <c s="995" r="CM89"/>
+      <c s="995" r="CN89"/>
+      <c s="995" r="CO89"/>
+      <c s="995" r="CP89"/>
+      <c s="995" r="CQ89"/>
+      <c s="995" r="CR89"/>
+      <c s="995" r="CS89"/>
+      <c s="995" r="CT89"/>
+      <c s="995" r="CU89"/>
+      <c s="995" r="CV89"/>
+      <c s="995" r="CW89"/>
+      <c s="995" r="CX89"/>
+      <c s="995" r="CY89"/>
+      <c s="995" r="CZ89"/>
+      <c s="995" r="DA89"/>
+      <c s="995" r="DB89"/>
+      <c s="995" r="DC89"/>
+      <c s="995" r="DD89"/>
+      <c s="995" r="DE89"/>
+      <c s="995" r="DF89"/>
+      <c s="995" r="DG89"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>